<commit_message>
hunt: extract 10 USTC SIST professors with full WebSearch enrichment
- 艾杨 (speech processing), 曹洋 (CV), 常晓军 (Embodied AI, 20000+ citations)
- 查正军 (CV/multimodal), 陈畅 (radar), 陈鹤 (postdoc)
- 陈力 (6G/ISAC, 优青), 陈绍青 (vibration control), 陈双武 (networking)
- 陈卫东 (radar, prof)
- Added auto-commit+push to SKILL.md Phase C
- Emails found for 8/10 via WebSearch
- Cross-linked 陈畅↔陈卫东 same lab
</commit_message>
<xml_diff>
--- a/docs/comparison.xlsx
+++ b/docs/comparison.xlsx
@@ -473,22 +473,22 @@
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="17.6" customWidth="1" min="2" max="2"/>
-    <col width="23.6" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="11.6" customWidth="1" min="4" max="4"/>
     <col width="11.6" customWidth="1" min="5" max="5"/>
     <col width="18.8" customWidth="1" min="6" max="6"/>
-    <col width="6.8" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
     <col width="17.6" customWidth="1" min="8" max="8"/>
     <col width="47.6" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="21.2" customWidth="1" min="11" max="11"/>
+    <col width="62" customWidth="1" min="10" max="10"/>
+    <col width="22.4" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="44" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="26" customWidth="1" min="18" max="18"/>
+    <col width="33.2" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -614,14 +614,26 @@
           <t>mainland_china</t>
         </is>
       </c>
-      <c r="G2" s="2" t="n"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>yangai@ustc.edu.cn</t>
+        </is>
+      </c>
       <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>语音合成, 语音增强, 语音分离, 音频编码, 音频质量评价</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>语音及语言信息处理国家工程研究中心</t>
+        </is>
+      </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>未知</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr"/>
@@ -634,12 +646,12 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12T23:30:00Z</t>
+          <t>2026-06-12T23:40:08.068167</t>
         </is>
       </c>
     </row>
@@ -674,10 +686,18 @@
           <t>mainland_china</t>
         </is>
       </c>
-      <c r="G3" s="2" t="n"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>forrest@ustc.edu.cn</t>
+        </is>
+      </c>
       <c r="H3" s="2" t="n"/>
       <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>计算机视觉, 深度学习, 图像处理, 排放源识别, 城市流预测</t>
+        </is>
+      </c>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
@@ -688,18 +708,20 @@
       <c r="N3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O3" s="2" t="n"/>
+      <c r="O3" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="P3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12T23:30:00Z</t>
+          <t>2026-06-12T23:40:08.068167</t>
         </is>
       </c>
     </row>
@@ -716,7 +738,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>教授 / 博士生导师 / 硕士生导师</t>
+          <t>讲席教授 / 博士生导师 / 硕士生导师</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -734,32 +756,50 @@
           <t>mainland_china</t>
         </is>
       </c>
-      <c r="G4" s="2" t="n"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>xjchang@ustc.edu.cn</t>
+        </is>
+      </c>
       <c r="H4" s="2" t="n"/>
       <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>具身智能, 多模态大模型, 类脑多模态智能, 计算机视觉, 绿色人工智能</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>具身智能与多模态学习实验室</t>
+        </is>
+      </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>未知</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr"/>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>欢迎有志于从事人工智能前沿研究的本科生、硕士生、博士生及实习生联系团队</t>
+        </is>
+      </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O4" s="2" t="n"/>
+      <c r="O4" s="2" t="n">
+        <v>35</v>
+      </c>
       <c r="P4" s="2" t="n">
         <v>0</v>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12T23:30:00Z</t>
+          <t>2026-06-12T23:40:08.068167</t>
         </is>
       </c>
     </row>
@@ -776,7 +816,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>高级工程师</t>
+          <t>正高级工程师</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -794,14 +834,26 @@
           <t>mainland_china</t>
         </is>
       </c>
-      <c r="G5" s="2" t="n"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>chench@ustc.edu.cn</t>
+        </is>
+      </c>
       <c r="H5" s="2" t="n"/>
       <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>射频微波系统, 雷达成像信号处理, 压缩感知与稀疏恢复, 滤波器设计, 涡旋电磁波超分辨成像</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>中国科学院电磁空间信息重点实验室</t>
+        </is>
+      </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>未知</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr"/>
@@ -814,12 +866,12 @@
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12T23:30:00Z</t>
+          <t>2026-06-12T23:40:08.068167</t>
         </is>
       </c>
     </row>
@@ -879,7 +931,7 @@
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12T23:30:00Z</t>
+          <t>2026-06-12T23:40:08.068167</t>
         </is>
       </c>
     </row>
@@ -896,7 +948,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>讲师</t>
+          <t>特任教授 / 副教授 / 博士生导师</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -914,14 +966,26 @@
           <t>mainland_china</t>
         </is>
       </c>
-      <c r="G7" s="2" t="n"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>chenli87@ustc.edu.cn</t>
+        </is>
+      </c>
       <c r="H7" s="2" t="n"/>
       <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>6G/5G无线通信, 通信感知计算一体化(ISAC), 分布式机器学习, 编码存储与计算, 边缘计算</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>无线光通信中国科学院重点实验室</t>
+        </is>
+      </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>未知</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr"/>
@@ -934,12 +998,12 @@
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12T23:30:00Z</t>
+          <t>2026-06-12T23:40:08.068167</t>
         </is>
       </c>
     </row>
@@ -974,10 +1038,18 @@
           <t>mainland_china</t>
         </is>
       </c>
-      <c r="G8" s="2" t="n"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>windcsq@ustc.edu.cn</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>振动主动控制, 磁悬浮隔振器, 自适应前馈控制, 自抗扰控制(ADRC)</t>
+        </is>
+      </c>
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr">
         <is>
@@ -994,12 +1066,12 @@
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12T23:30:00Z</t>
+          <t>2026-06-12T23:40:08.068167</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1088,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>（待确认）</t>
+          <t>副教授 / 副研究员</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1034,14 +1106,26 @@
           <t>mainland_china</t>
         </is>
       </c>
-      <c r="G9" s="2" t="n"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>chensw@ustc.edu.cn</t>
+        </is>
+      </c>
       <c r="H9" s="2" t="n"/>
       <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>智能网络, 智能计算, 网络安全, 多媒体通信, 工业互联网</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>未来网络安徽省重点实验室</t>
+        </is>
+      </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>未知</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr"/>
@@ -1054,12 +1138,12 @@
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12T23:30:00Z</t>
+          <t>2026-06-12T23:40:08.068167</t>
         </is>
       </c>
     </row>
@@ -1076,7 +1160,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>教授</t>
+          <t>教授 / 博士生导师</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1094,14 +1178,30 @@
           <t>mainland_china</t>
         </is>
       </c>
-      <c r="G10" s="2" t="n"/>
-      <c r="H10" s="2" t="n"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>wdchen@ustc.edu.cn</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>0551-63601303</t>
+        </is>
+      </c>
       <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>微波毫米波系统, 雷达信号与信息处理, 微波凝视关联成像, 分布式雷达超分辨成像</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>中国科学院电磁空间信息重点实验室</t>
+        </is>
+      </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>未知</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr"/>
@@ -1114,12 +1214,12 @@
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12T23:30:00Z</t>
+          <t>2026-06-12T23:40:08.068167</t>
         </is>
       </c>
     </row>
@@ -1320,7 +1420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1360,25 +1460,167 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>语音及语言信息处理国家工程研究中心</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>艾杨</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>中国科学技术大学</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>web_search</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>具身智能与多模态学习实验室</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>常晓军</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>中国科学技术大学</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>web_search</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>中国科学院电磁空间信息重点实验室</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>陈畅</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>中国科学技术大学</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>web_search</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>无线光通信中国科学院重点实验室</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>陈力</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>中国科学技术大学</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>web_search</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>http://woc-lab.ustc.edu.cn</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>未来网络安徽省重点实验室</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>陈双武</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>中国科学技术大学</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>web_search</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>中国科学院电磁空间信息重点实验室</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>陈卫东</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>中国科学技术大学</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>web_search</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
           <t>类脑智能技术及应用国家工程实验室</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>查正军</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>中国科学技术大学</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>homepage_bio</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
hunt: add paper details for 查正军(15 papers) and 常晓军(3 papers)
- 查正军: 15 papers (CVPR/ICLR/ICML/ECCV/AAAI/ACL/SIGGRAPH/MM + PAMI/IJCV), 7 inferred students
- 常晓军: 3 PAMI papers (2024), 3 inferred students
- Paper source: WebSearch (Google Scholar blocked, DBLP blocked, Semantic Scholar empty)
- Known limitation: WebFetch blocked for scholar.google.com, dblp.org, faculty.ustc.edu.cn
  Paper data depends on WebSearch results which vary by professor prominence
</commit_message>
<xml_diff>
--- a/docs/comparison.xlsx
+++ b/docs/comparison.xlsx
@@ -14,6 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'对比总表'!$A$1:$R$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'论文列表'!$A$1:$H$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -784,17 +785,17 @@
         </is>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O4" s="2" t="n">
         <v>35</v>
       </c>
       <c r="P4" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
@@ -1278,15 +1279,15 @@
       </c>
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="O11" s="2" t="n"/>
       <c r="P11" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr">
@@ -1323,52 +1324,675 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>导师</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>论文标题</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>作者</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>期刊/会议</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>年份</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>类型</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>引用数</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>常晓军</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Simple Primitives With Feasibility- and Contextuality-Dependence for Open-World Compositional Zero-Shot Learning</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Zhe Liu, Yun Li, Lina Yao, Xiaojun Chang, Wei Fang, Xiaojun Wu, Abdulmotaleb El-Saddik</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Trans. PAMI</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>journal</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>常晓军</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>DNA Family: Boosting Weight-Sharing NAS With Block-Wise Supervisions</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Guangrun Wang, Changlin Li, Liuchun Yuan, Jiefeng Peng, Xiaoyu Xian, Xiaodan Liang, Xiaojun Chang, Liang Lin</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Trans. PAMI</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>journal</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>常晓军</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Semantics-Guided Contrastive Network for Zero-Shot Object Detection</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Caixia Yan, Xiaojun Chang, Minnan Luo, Huan Liu, Xiaoqin Zhang, Qinghua Zheng</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Trans. PAMI</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>journal</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>WeMMU: Enhanced Bridging of Vision-Language Models and Diffusion Models via Noisy Query Tokens</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Jian Yang, Dacheng Yin, Xiao He, Yong Li, Fengyun Rao, Jing Lyu, Wei Zhai, Yang Cao, Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>arXiv</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>LEMON: Learning 3D Human-Object Interaction Relation from 2D Images</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Yuhang Yang, Wei Zhai, Hongchen Luo, Yang Cao, Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>CVPR</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Prompt-Enhanced Multiple Instance Learning for Weakly Supervised Video Anomaly Detection</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Junxi Chen, Liang Li, Li Su, Qingming Huang, Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>CVPR</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>HomoFormer: Homogenized Transformer for Image Shadow Removal</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Jie Xiao, Xueyang Fu, Yurui Zhu, Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>CVPR</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>DreamClean: Restoring Clean Image Using Deep Diffusion Prior</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Jie Xiao, Ruili Feng, Han Zhang, Zhiheng Liu, Zhantao Yang, Yurui Zhu, Xueyang Fu, Kai Zhu, Yu Liu, Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>ICLR</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>CCM: Real-Time Controllable Visual Content Creation Using Text-to-Image Consistency Models</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Jie Xiao, Kai Zhu, Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>ICML</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Event-Adapted Video Super-Resolution</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Zeyu Xiao, Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>ECCV</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Motion Aware Event Representation-Driven Image Deblurring</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Zhijing Sun, Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>ECCV</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Neuromorphic Event Signal-Driven Network for Video De-raining</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>AAAI</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Context-aware Difference Distilling for Multi-change Captioning</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Yunbin Tu, Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>ACL</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>I2V-Adapter: A General Image-to-Video Adapter for Diffusion Models</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>SIGGRAPH</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Cross-Modal Semantic Alignment Learning for Text-Based Person Search</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>ACM Multimedia</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Background Activation Suppression for Weakly Supervised Object Localization and Semantic Segmentation</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>IJCV</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>journal</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>SMART: Syntax-Calibrated Multi-Aspect Relation Transformer for Change Captioning</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Trans. PAMI</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>journal</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Inductive State-Relabeling Adversarial Active Learning</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Trans. PAMI</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>journal</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:H19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1379,33 +2003,290 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>导师</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>学生姓名</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>推断来源</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>作为一作论文数</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>一作论文列表</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>常晓军</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Caixia Yan</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>论文一作反推</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Trans. PAMI 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>常晓军</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Guangrun Wang</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>论文一作反推</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Trans. PAMI 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>常晓军</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Zhe Liu</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>论文一作反推</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Trans. PAMI 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Jian Yang</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>论文一作反推</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>arXiv 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Jie Xiao</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>论文一作反推</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>CVPR 2024, ICLR 2024, ICML 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Junxi Chen</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>论文一作反推</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>CVPR 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Yuhang Yang</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>论文一作反推</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>CVPR 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Yunbin Tu</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>论文一作反推</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>ACL 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Zeyu Xiao</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>论文一作反推</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>ECCV 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Zhijing Sun</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>论文一作反推</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>ECCV 2024</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ui: enhance paper display - year sorting, research tags from titles, source badges
</commit_message>
<xml_diff>
--- a/docs/comparison.xlsx
+++ b/docs/comparison.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'对比总表'!$A$1:$R$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'论文列表'!$A$1:$H$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'论文列表'!$A$1:$H$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -639,7 +639,7 @@
       </c>
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2" s="2" t="n"/>
       <c r="P2" s="2" t="n">
@@ -652,7 +652,7 @@
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12T23:40:08.068167</t>
+          <t>2026-06-13T00:14:03.075825</t>
         </is>
       </c>
     </row>
@@ -1324,7 +1324,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1382,36 +1382,34 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>常晓军</t>
+          <t>艾杨</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Simple Primitives With Feasibility- and Contextuality-Dependence for Open-World Compositional Zero-Shot Learning</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Zhe Liu, Yun Li, Lina Yao, Xiaojun Chang, Wei Fang, Xiaojun Wu, Abdulmotaleb El-Saddik</t>
-        </is>
-      </c>
+          <t>{'value': 'Yang-Baxter Invariants for Line Configurations'}</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>IEEE Trans. PAMI</t>
+          <t>{'value': 'Discret. Comput. Geom. 1996'}</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>2024</v>
+        <v>8204</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>journal</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" s="2" t="inlineStr"/>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>https://ieeexplore.ieee.org/author/37086348873</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1421,12 +1419,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>DNA Family: Boosting Weight-Sharing NAS With Block-Wise Supervisions</t>
+          <t>Simple Primitives With Feasibility- and Contextuality-Dependence for Open-World Compositional Zero-Shot Learning</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Guangrun Wang, Changlin Li, Liuchun Yuan, Jiefeng Peng, Xiaoyu Xian, Xiaodan Liang, Xiaojun Chang, Liang Lin</t>
+          <t>Zhe Liu, Yun Li, Lina Yao, Xiaojun Chang, Wei Fang, Xiaojun Wu, Abdulmotaleb El-Saddik</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1445,7 +1443,11 @@
       <c r="G3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?user=8suupocAAAAJ</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1455,12 +1457,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Semantics-Guided Contrastive Network for Zero-Shot Object Detection</t>
+          <t>DNA Family: Boosting Weight-Sharing NAS With Block-Wise Supervisions</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Caixia Yan, Xiaojun Chang, Minnan Luo, Huan Liu, Xiaoqin Zhang, Qinghua Zheng</t>
+          <t>Guangrun Wang, Changlin Li, Liuchun Yuan, Jiefeng Peng, Xiaoyu Xian, Xiaodan Liang, Xiaojun Chang, Liang Lin</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1479,41 +1481,49 @@
       <c r="G4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?user=8suupocAAAAJ</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>查正军</t>
+          <t>常晓军</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>WeMMU: Enhanced Bridging of Vision-Language Models and Diffusion Models via Noisy Query Tokens</t>
+          <t>Semantics-Guided Contrastive Network for Zero-Shot Object Detection</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Jian Yang, Dacheng Yin, Xiao He, Yong Li, Fengyun Rao, Jing Lyu, Wei Zhai, Yang Cao, Zhengjun Zha</t>
+          <t>Caixia Yan, Xiaojun Chang, Minnan Luo, Huan Liu, Xiaoqin Zhang, Qinghua Zheng</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>arXiv</t>
+          <t>IEEE Trans. PAMI</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>preprint</t>
+          <t>journal</t>
         </is>
       </c>
       <c r="G5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?user=8suupocAAAAJ</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1523,31 +1533,31 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>LEMON: Learning 3D Human-Object Interaction Relation from 2D Images</t>
+          <t>WeMMU: Enhanced Bridging of Vision-Language Models and Diffusion Models via Noisy Query Tokens</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Yuhang Yang, Wei Zhai, Hongchen Luo, Yang Cao, Zhengjun Zha</t>
+          <t>Jian Yang, Dacheng Yin, Xiao He, Yong Li, Fengyun Rao, Jing Lyu, Wei Zhai, Yang Cao, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>CVPR</t>
+          <t>arXiv</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>conference</t>
+          <t>preprint</t>
         </is>
       </c>
       <c r="G6" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1557,12 +1567,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Prompt-Enhanced Multiple Instance Learning for Weakly Supervised Video Anomaly Detection</t>
+          <t>LEMON: Learning 3D Human-Object Interaction Relation from 2D Images</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Junxi Chen, Liang Li, Li Su, Qingming Huang, Zhengjun Zha</t>
+          <t>Yuhang Yang, Wei Zhai, Hongchen Luo, Yang Cao, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1581,7 +1591,7 @@
       <c r="G7" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1591,12 +1601,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>HomoFormer: Homogenized Transformer for Image Shadow Removal</t>
+          <t>Prompt-Enhanced Multiple Instance Learning for Weakly Supervised Video Anomaly Detection</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Jie Xiao, Xueyang Fu, Yurui Zhu, Zhengjun Zha</t>
+          <t>Junxi Chen, Liang Li, Li Su, Qingming Huang, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1615,7 +1625,7 @@
       <c r="G8" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1625,17 +1635,17 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>DreamClean: Restoring Clean Image Using Deep Diffusion Prior</t>
+          <t>HomoFormer: Homogenized Transformer for Image Shadow Removal</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Jie Xiao, Ruili Feng, Han Zhang, Zhiheng Liu, Zhantao Yang, Yurui Zhu, Xueyang Fu, Kai Zhu, Yu Liu, Zhengjun Zha</t>
+          <t>Jie Xiao, Xueyang Fu, Yurui Zhu, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>ICLR</t>
+          <t>CVPR</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
@@ -1649,7 +1659,7 @@
       <c r="G9" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1659,17 +1669,17 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>CCM: Real-Time Controllable Visual Content Creation Using Text-to-Image Consistency Models</t>
+          <t>DreamClean: Restoring Clean Image Using Deep Diffusion Prior</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Jie Xiao, Kai Zhu, Zhengjun Zha</t>
+          <t>Jie Xiao, Ruili Feng, Han Zhang, Zhiheng Liu, Zhantao Yang, Yurui Zhu, Xueyang Fu, Kai Zhu, Yu Liu, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>ICML</t>
+          <t>ICLR</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
@@ -1683,7 +1693,7 @@
       <c r="G10" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1693,17 +1703,17 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Event-Adapted Video Super-Resolution</t>
+          <t>CCM: Real-Time Controllable Visual Content Creation Using Text-to-Image Consistency Models</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Zeyu Xiao, Zhengjun Zha</t>
+          <t>Jie Xiao, Kai Zhu, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>ECCV</t>
+          <t>ICML</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
@@ -1717,7 +1727,7 @@
       <c r="G11" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1727,12 +1737,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Motion Aware Event Representation-Driven Image Deblurring</t>
+          <t>Event-Adapted Video Super-Resolution</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Zhijing Sun, Zhengjun Zha</t>
+          <t>Zeyu Xiao, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1751,7 +1761,7 @@
       <c r="G12" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1761,17 +1771,17 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Neuromorphic Event Signal-Driven Network for Video De-raining</t>
+          <t>Motion Aware Event Representation-Driven Image Deblurring</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Zhengjun Zha</t>
+          <t>Zhijing Sun, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>AAAI</t>
+          <t>ECCV</t>
         </is>
       </c>
       <c r="E13" s="2" t="n">
@@ -1785,7 +1795,7 @@
       <c r="G13" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1795,17 +1805,17 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Context-aware Difference Distilling for Multi-change Captioning</t>
+          <t>Neuromorphic Event Signal-Driven Network for Video De-raining</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Yunbin Tu, Zhengjun Zha</t>
+          <t>Zhengjun Zha</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>ACL</t>
+          <t>AAAI</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
@@ -1819,7 +1829,7 @@
       <c r="G14" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1829,17 +1839,17 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>I2V-Adapter: A General Image-to-Video Adapter for Diffusion Models</t>
+          <t>Context-aware Difference Distilling for Multi-change Captioning</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Zhengjun Zha</t>
+          <t>Yunbin Tu, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>SIGGRAPH</t>
+          <t>ACL</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
@@ -1853,7 +1863,7 @@
       <c r="G15" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1863,7 +1873,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Cross-Modal Semantic Alignment Learning for Text-Based Person Search</t>
+          <t>I2V-Adapter: A General Image-to-Video Adapter for Diffusion Models</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1873,7 +1883,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>ACM Multimedia</t>
+          <t>SIGGRAPH</t>
         </is>
       </c>
       <c r="E16" s="2" t="n">
@@ -1887,7 +1897,7 @@
       <c r="G16" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1897,7 +1907,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Background Activation Suppression for Weakly Supervised Object Localization and Semantic Segmentation</t>
+          <t>Cross-Modal Semantic Alignment Learning for Text-Based Person Search</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1907,7 +1917,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>IJCV</t>
+          <t>ACM Multimedia</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
@@ -1915,13 +1925,13 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>journal</t>
+          <t>conference</t>
         </is>
       </c>
       <c r="G17" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1931,7 +1941,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>SMART: Syntax-Calibrated Multi-Aspect Relation Transformer for Change Captioning</t>
+          <t>Background Activation Suppression for Weakly Supervised Object Localization and Semantic Segmentation</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1941,7 +1951,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>IEEE Trans. PAMI</t>
+          <t>IJCV</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
@@ -1955,7 +1965,7 @@
       <c r="G18" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1965,7 +1975,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Inductive State-Relabeling Adversarial Active Learning</t>
+          <t>SMART: Syntax-Calibrated Multi-Aspect Relation Transformer for Change Captioning</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1989,10 +1999,44 @@
       <c r="G19" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Inductive State-Relabeling Adversarial Active Learning</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Trans. PAMI</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>journal</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H19"/>
+  <autoFilter ref="A1:H20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
papers: multi-channel collection (DBLP+OpenReview+arXiv) for 164 USTC professors - 91 papers from 10 professors
- DBLP: most papers, but severe name ambiguity for common Chinese names
- OpenReview: ML conference papers only
- arXiv: preprints
- Known limitation: ~90% of professors have no unique DBLP match
- Recommendation: WebSearch as primary, APIs as supplement
</commit_message>
<xml_diff>
--- a/docs/comparison.xlsx
+++ b/docs/comparison.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'对比总表'!$A$1:$R$165</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'论文列表'!$A$1:$H$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'论文列表'!$A$1:$H$110</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -695,7 +695,7 @@
       </c>
       <c r="M3" s="2" t="inlineStr"/>
       <c r="N3" s="2" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="O3" s="2" t="n"/>
       <c r="P3" s="2" t="n">
@@ -703,12 +703,12 @@
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T00:14:03.075825</t>
+          <t>2026-06-13T00:47:30.891658</t>
         </is>
       </c>
     </row>
@@ -763,7 +763,7 @@
       </c>
       <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O4" s="2" t="n">
         <v>13</v>
@@ -773,12 +773,12 @@
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12T23:40:08.068167</t>
+          <t>2026-06-13T00:47:30.928569</t>
         </is>
       </c>
     </row>
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="N6" s="2" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="O6" s="2" t="n">
         <v>35</v>
@@ -907,12 +907,12 @@
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12T23:40:08.068167</t>
+          <t>2026-06-13T00:47:30.938516</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="M8" s="2" t="inlineStr"/>
       <c r="N8" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O8" s="2" t="n"/>
       <c r="P8" s="2" t="n">
@@ -1039,12 +1039,12 @@
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12T23:40:08.068167</t>
+          <t>2026-06-13T00:47:30.938114</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O9" s="2" t="n"/>
       <c r="P9" s="2" t="n">
@@ -1099,12 +1099,12 @@
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12T23:40:08.068167</t>
+          <t>2026-06-13T00:47:30.907309</t>
         </is>
       </c>
     </row>
@@ -1163,7 +1163,7 @@
       </c>
       <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O10" s="2" t="n"/>
       <c r="P10" s="2" t="n">
@@ -1176,7 +1176,7 @@
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12T23:40:08.068167</t>
+          <t>2026-06-13T00:47:35.601597</t>
         </is>
       </c>
     </row>
@@ -1287,7 +1287,7 @@
       </c>
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O12" s="2" t="n"/>
       <c r="P12" s="2" t="n">
@@ -1300,7 +1300,7 @@
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12T23:40:08.068167</t>
+          <t>2026-06-13T00:47:35.504227</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1359,7 @@
       </c>
       <c r="M13" s="2" t="inlineStr"/>
       <c r="N13" s="2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="O13" s="2" t="n"/>
       <c r="P13" s="2" t="n">
@@ -1367,12 +1367,12 @@
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12T23:40:08.068167</t>
+          <t>2026-06-13T00:47:35.874843</t>
         </is>
       </c>
     </row>
@@ -1435,7 +1435,7 @@
       </c>
       <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O14" s="2" t="n"/>
       <c r="P14" s="2" t="n">
@@ -1443,12 +1443,12 @@
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12T23:40:08.068167</t>
+          <t>2026-06-13T00:47:35.883136</t>
         </is>
       </c>
     </row>
@@ -9119,7 +9119,7 @@
       </c>
       <c r="M152" s="2" t="inlineStr"/>
       <c r="N152" s="2" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="O152" s="2" t="n"/>
       <c r="P152" s="2" t="n">
@@ -9132,7 +9132,7 @@
       </c>
       <c r="R152" s="2" t="inlineStr">
         <is>
-          <t>2026-06-12T00:00:00Z</t>
+          <t>2026-06-13T00:47:35.728993</t>
         </is>
       </c>
     </row>
@@ -9888,7 +9888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -9978,629 +9978,3509 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>常晓军</t>
+          <t>艾杨</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Simple Primitives With Feasibility- and Contextuality-Dependence for Open-World Compositional Zero-Shot Learning</t>
+          <t>Beyond WER: A Paired Acoustic Stress Test for Ambient Clinical Scribes</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Zhe Liu, Yun Li, Lina Yao, Xiaojun Chang, Wei Fang, Xiaojun Wu, Abdulmotaleb El-Saddik</t>
+          <t>Xiao-Hang Jiang, Han-Jie Guo, Ying-Si Liang, Yang Ai, Zhen-Hua Ling, Lei Jiang, Zhi-Yang He</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>IEEE Trans. PAMI</t>
+          <t>Accepted to INTERSPEECH 2026</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>journal</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?user=8suupocAAAAJ</t>
-        </is>
-      </c>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>常晓军</t>
+          <t>艾杨</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>DNA Family: Boosting Weight-Sharing NAS With Block-Wise Supervisions</t>
+          <t>VoCodec: A Low-bitrate Streamable Neural Speech Codec with Voicing-driven Quantization</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Guangrun Wang, Changlin Li, Liuchun Yuan, Jiefeng Peng, Xiaoyu Xian, Xiaodan Liang, Xiaojun Chang, Liang Lin</t>
+          <t>Xiao-Hang Jiang, Yang Ai, Rui-Chen Zheng, Li-Rong Dai, Zhen-Hua Ling, Ji Wu</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>IEEE Trans. PAMI</t>
+          <t>Accepted to INTERSPEECH 2026</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>journal</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?user=8suupocAAAAJ</t>
-        </is>
-      </c>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>常晓军</t>
+          <t>艾杨</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Semantics-Guided Contrastive Network for Zero-Shot Object Detection</t>
+          <t>An Ultra-Low-Bitrate Neural Speech Codec with Plain-to-Pseudo Synergistic Vector Quantization</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Caixia Yan, Xiaojun Chang, Minnan Luo, Huan Liu, Xiaoqin Zhang, Qinghua Zheng</t>
+          <t>Xiao-Hang Jiang, Yang Ai, Fei Liu, Rui-Chen Zheng, Jian-Qing Gao, Zhen-Hua Ling, Ji Wu</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>IEEE Trans. PAMI</t>
+          <t>Accepted to INTERSPEECH 2026</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>journal</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>https://scholar.google.com/citations?user=8suupocAAAAJ</t>
-        </is>
-      </c>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>查正军</t>
+          <t>艾杨</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>WeMMU: Enhanced Bridging of Vision-Language Models and Diffusion Models via Noisy Query Tokens</t>
+          <t>UniVocal: Unified Speech-Singing Code-Switching Synthesis</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Jian Yang, Dacheng Yin, Xiao He, Yong Li, Fengyun Rao, Jing Lyu, Wei Zhai, Yang Cao, Zhengjun Zha</t>
+          <t>Yufei Shi, Qian Chen, Wen Wang, Xiangang Li, Zhen-Hua Ling, Yang Ai</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>arXiv</t>
+          <t>accepted by ACL 2026</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>preprint</t>
         </is>
       </c>
-      <c r="G6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>查正军</t>
+          <t>艾杨</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>LEMON: Learning 3D Human-Object Interaction Relation from 2D Images</t>
+          <t>CFMDCTCodec: A Low-Bitrate Neural Speech Codec with Noise-Prior-aware Conditional Flow Matching for MDCT-Spectral Enhancement</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Yuhang Yang, Wei Zhai, Hongchen Luo, Yang Cao, Zhengjun Zha</t>
+          <t>Xiao-Hang Jiang, Yang Ai, Hui-Peng Du, Zhen-Hua Ling, Ji Wu</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>CVPR</t>
+          <t>Accepted by IEEE Transactions on Audio, Speech and Language Processing</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>conference</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="2" t="n"/>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>查正军</t>
+          <t>艾杨</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Prompt-Enhanced Multiple Instance Learning for Weakly Supervised Video Anomaly Detection</t>
+          <t>Ultra-Low-Bitrate Mel-Spectrogram-based Neural Speech Coding with Flow-Matching-based Refinement and Vocoding-driven Reconstruction</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Junxi Chen, Liang Li, Li Su, Qingming Huang, Zhengjun Zha</t>
+          <t>Hui-Peng Du, Yang Ai, Xiao-Hang Jiang, Yuan Tian, Zhen-Hua Ling</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>CVPR</t>
+          <t>Published at IEEE/ACM Transactions on Audio, Speech, and Language Processing</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>conference</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="2" t="n"/>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>查正军</t>
+          <t>艾杨</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>HomoFormer: Homogenized Transformer for Image Shadow Removal</t>
+          <t>LatentFlowSR: High-Fidelity Audio Super-Resolution via Noise-Robust Latent Flow Matching</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Jie Xiao, Xueyang Fu, Yurui Zhu, Zhengjun Zha</t>
+          <t>Fei Liu, Yang Ai, Hui-Peng Du, Yu-Fei Shi, Zhen-Hua Ling</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>CVPR</t>
+          <t>arXiv preprint</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>conference</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="2" t="n"/>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>查正军</t>
+          <t>艾杨</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>DreamClean: Restoring Clean Image Using Deep Diffusion Prior</t>
+          <t>ParaGSE: Parallel Generative Speech Enhancement with Group-Vector-Quantization-based Neural Speech Codec</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Jie Xiao, Ruili Feng, Han Zhang, Zhiheng Liu, Zhantao Yang, Yurui Zhu, Xueyang Fu, Kai Zhu, Yu Liu, Zhengjun Zha</t>
+          <t>Fei Liu, Yang Ai</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>ICLR</t>
+          <t>Accepted by ICASSP 2026</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>conference</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="2" t="n"/>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>查正军</t>
+          <t>艾杨</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>CCM: Real-Time Controllable Visual Content Creation Using Text-to-Image Consistency Models</t>
+          <t>CodeSep: Low-Bitrate Codec-Driven Speech Separation with Base-Token Disentanglement and Auxiliary-Token Serial Prediction</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Jie Xiao, Kai Zhu, Zhengjun Zha</t>
+          <t>Hui-Peng Du, Yang Ai, Xiao-Hang Jiang, Rui-Chen Zheng, Zhen-Hua Ling</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>ICML</t>
+          <t>Accepted by ICASSP 2026</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>conference</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="2" t="n"/>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>查正军</t>
+          <t>艾杨</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Event-Adapted Video Super-Resolution</t>
+          <t>DAIEN-TTS: Disentangled Audio Infilling for Environment-Aware Text-to-Speech Synthesis</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Zeyu Xiao, Zhengjun Zha</t>
+          <t>Ye-Xin Lu, Yu Gu, Kun Wei, Hui-Peng Du, Yang Ai, Zhen-Hua Ling</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>ECCV</t>
+          <t>Accepted by ICASSP 2026</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>conference</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="2" t="n"/>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>查正军</t>
+          <t>曹洋</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Motion Aware Event Representation-Driven Image Deblurring</t>
+          <t>Back on Track: Aligning Rewards and States for Reasoning in Diffusion Large Language Models</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Zhijing Sun, Zhengjun Zha</t>
+          <t>Yawen Shao, Jie Xiao, Kai Zhu, Yu Liu, Hongchen Luo, Xueyang Fu, Yang Cao, Wei Zhai, Zheng-Jun Zha</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>ECCV</t>
+          <t>arXiv preprint</t>
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>conference</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="2" t="n"/>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>查正军</t>
+          <t>曹洋</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Neuromorphic Event Signal-Driven Network for Video De-raining</t>
+          <t>Beyond Fixed Rounds: Data-Free Early Stopping for Practical Federated Learning</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Zhengjun Zha</t>
+          <t>Youngjoon Lee, Hyukjoon Lee, Seungrok Jung, Andy Luo, Jinu Gong, Yang Cao, Joonhyuk Kang</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>AAAI</t>
+          <t>Under Review</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>conference</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="2" t="n"/>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>查正军</t>
+          <t>曹洋</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Context-aware Difference Distilling for Multi-change Captioning</t>
+          <t>Near-Field Coupling of Polypropylene Dielectric Waveguide Routed Near PCB Board at Terahertz Frequencies</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Yunbin Tu, Zhengjun Zha</t>
+          <t>Wenbo Liu, Jiabiao Zhao, Kefeng Huang, Peian Li, Boquan Xu, Yang Cao, Weidong Hu, Jianjun Ma</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>ACL</t>
+          <t>Submitted to Nano Communication Networks</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>conference</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="2" t="n"/>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>查正军</t>
+          <t>曹洋</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>I2V-Adapter: A General Image-to-Video Adapter for Diffusion Models</t>
+          <t>CLFEC: A New Task for Unified Linguistic and Factual Error Correction in paragraph-level Chinese Professional Writing</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Zhengjun Zha</t>
+          <t>Jian Kai, Zidong Zhang, Jiwen Chen, Zhengxiang Wu, Songtao Sun, Fuyang Li, Yang Cao, Qiang Liu</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>SIGGRAPH</t>
+          <t>arXiv preprint</t>
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>conference</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="2" t="n"/>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>查正军</t>
+          <t>曹洋</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Cross-Modal Semantic Alignment Learning for Text-Based Person Search</t>
+          <t>Stepwise Reasoning Enhancement for LLMs via External Subgraph Generation</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Zhengjun Zha</t>
+          <t>Xin Zhang, Yang Cao, Baoxing Wu, Kai Song, Siying Li</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>ACM Multimedia</t>
+          <t>arXiv preprint</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>conference</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="2" t="n"/>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>查正军</t>
+          <t>曹洋</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Background Activation Suppression for Weakly Supervised Object Localization and Semantic Segmentation</t>
+          <t>SeClaw: Spec-Driven Security Task Synthesis for Evaluating Autonomous Agents</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Zhengjun Zha</t>
+          <t>Hao Cheng, Changtao Miao, Tianle Song, Yin Wu, He Liu, Erjia Xiao, Junchi Chen, Xiaoyu Shi, Yichi Wang, Jing Yang, Taowen Wang, Jinhao Duan, Mengshu Sun, Peiyan Dong, Xuan Shen, Yang Cao, Renjing Xu, Kaidi Xu, Jindong Gu, Bo Zhang, Jize Zhang, Chenhao Lin, Philip Torr, Chao Shen</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>IJCV</t>
+          <t>arXiv preprint</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>journal</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="2" t="n"/>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>查正军</t>
+          <t>曹洋</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>SMART: Syntax-Calibrated Multi-Aspect Relation Transformer for Change Captioning</t>
+          <t>Vector Linking via Cross-Model Local Isometric Consistency</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Zhengjun Zha</t>
+          <t>Ziying Chen, Yang Cao, He Sun, Beining Yang, Tianjian Yang</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>IEEE Trans. PAMI</t>
+          <t>Accepted at ICML 2026</t>
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>journal</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="2" t="n"/>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>曹洋</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Multi-Adapter Representation Interventions via Energy Calibration</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Manjiang Yu, Hongji Li, Junwei Chen, Xue Li, Priyanka Singh, Yang Cao, Lijie Hu</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by ICML 2026</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>曹洋</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Tail-Aware HiFloat4: W4A4 Post-Training Quantization for Wan2.2</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Zhanfeng Feng, Shuai Guo, Xin Di, Long Peng, Yang Cao, Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>曹洋</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>RAD: A Dataset and Benchmark for Real-Life Anomaly Detection with Robotic Observations</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Kaichen Zhou, Xinhai Chang, Taewhan Kim, Jiadong Zhang, Yang Cao, Chufei Peng, Fangneng Zhan, Hao Zhao, Hao Dong, Kai Ming Ting, Ye Zhu</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>常晓军</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>See, Plan, Rewind: Progress-Aware Vision-Language-Action Models for Robust Robotic Manipulation</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Tingjun Dai, Mingfei Han, Tingwen Du, Zhiheng Liu, Zihao Zhang, Zhihui Li, Salman Khan, Jun Yu, Xiaojun Chang</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Suggested to CVPR Findings. https://tingjundai.github.io/SPRVLA/</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>常晓军</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>SRC-Flow: Compact Semantic Representations Enable Normalizing Flows for Image Generation</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Longtao Jiang, Jianmin Bao, Zhendong Wang, Xin Tao, Pengfei Wan, Zhihui Li, Xiaojun Chang</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>常晓军</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Zero-Shot Neural Network Evaluation with Sample-Wise Activation Patterns</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Yameng Peng, Andy Song, HaythamM. Fayek, Vic Ciesielski, Xiaojun Chang</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by IEEE Transactions on Pattern Analysis and Machine Intelligence. This</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>常晓军</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Progressive Online Video Understanding with Evidence-Aligned Timing and Transparent Decisions</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Kecheng Zhang, Zongxin Yang, Mingfei Han, Haihong Hao, Yunzhi Zhuge, Changlin Li, Junhan Zhao, Zhihui Li, Xiaojun Chang</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>常晓军</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Measuring Social Bias in Vision-Language Models with Face-Only Counterfactuals from Real Photos</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Haodong Chen, Qiang Huang, Jiaqi Zhao, Qiuping Jiang, Xiaojun Chang, Jun Yu</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>18 pages, 18 figures, and 3 tables</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="n"/>
+      <c r="H27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>常晓军</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>A1: A Fully Transparent Open-Source, Adaptive and Efficient Truncated Vision-Language-Action Model</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Kaidong Zhang, Jian Zhang, Rongtao Xu, Yu Sun, Shuoshuo Xue, Youpeng Wen, Xiaoyu Guo, Minghao Guo, Weijia Liufu, Liu Zihou, Kangyi Ji, Yangsong Zhang, Jiarun Zhu, Jingzhi Liu, Zihang Li, Ruiyi Chen, Meng Cao, Jingming Zhang, Shen Zhao, Xiaojun Chang, Feng Zheng, Ivan Laptev, Xiaodan Liang</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="n"/>
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>常晓军</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>LatentPilot: Scene-Aware Vision-and-Language Navigation by Dreaming Ahead with Latent Visual Reasoning</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Haihong Hao, Lei Chen, Mingfei Han, Changlin Li, Dong An, Yuqiang Yang, Zhihui Li, Xiaojun Chang</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Project page:https://abdd.top/latentpilot/</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="n"/>
+      <c r="H29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>常晓军</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>FACE-net: Factual Calibration and Emotion Augmentation for Retrieval-enhanced Emotional Video Captioning</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Weidong Chen, Cheng Ye, Zhendong Mao, Peipei Song, Xinyan Liu, Lei Zhang, Xiaojun Chang, Yongdong Zhang</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Submitted to TPAMI. 16 pages, 9 figures</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="n"/>
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>常晓军</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>EmoVerse: A MLLMs-Driven Emotion Representation Dataset for Interpretable Visual Emotion Analysis</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Yijie Guo, Dexiang Hong, Weidong Chen, Zihan She, Cheng Ye, Xiaojun Chang, Zhendong Mao</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>11 pages, 7 figures. This is a preprint version of a paper submitted to CVPR 202</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="n"/>
+      <c r="H31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>常晓军</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>CARE What Fails: Contrastive Anchored-REflection for Verifiable Multimodal Reasoning</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Yongxin Wang, Zhicheng Yang, Meng Cao, Mingfei Han, Haokun Lin, Yingying Zhu, Xiaojun Chang, Xiaodan Liang</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="n"/>
+      <c r="H32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>常晓军</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Simple Primitives With Feasibility- and Contextuality-Dependence for Open-World Compositional Zero-Shot Learning</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Zhe Liu, Yun Li, Lina Yao, Xiaojun Chang, Wei Fang, Xiaojun Wu, Abdulmotaleb El-Saddik</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Trans. PAMI</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>journal</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?user=8suupocAAAAJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>常晓军</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>DNA Family: Boosting Weight-Sharing NAS With Block-Wise Supervisions</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Guangrun Wang, Changlin Li, Liuchun Yuan, Jiefeng Peng, Xiaoyu Xian, Xiaodan Liang, Xiaojun Chang, Liang Lin</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Trans. PAMI</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>journal</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?user=8suupocAAAAJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>常晓军</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Semantics-Guided Contrastive Network for Zero-Shot Object Detection</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Caixia Yan, Xiaojun Chang, Minnan Luo, Huan Liu, Xiaoqin Zhang, Qinghua Zheng</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Trans. PAMI</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>journal</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>https://scholar.google.com/citations?user=8suupocAAAAJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>陈畅</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Probing Multimodal Large Language Models on Cognitive Biases in Chinese Short-Video Misinformation</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Jen-tse Huang, Chang Chen, Shiyang Lai, Wenxuan Wang, Michelle R. Kaufman, Mark Dredze</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Accepted to ACL 2026 (Findings)</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="n"/>
+      <c r="H36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>陈畅</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Before the Shutter: Aesthetic and Actionable Portrait Photography Planning in 3D Scenes</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Ruixiang Jiang, Chang Wen Chen</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="n"/>
+      <c r="H37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>陈畅</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>FlashEvolve: Accelerating Agent Self-Evolution with Asynchronous Stage Orchestration</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Zhengding Hu, Mingge Lu, Zhen Wang, Jixuan Ruan, Chang Chen, Zaifeng Pan, Yue Guan, Ruiyi Wang, Zhongkai Yu, Chao Zhang, Yufei Ding</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="n"/>
+      <c r="H38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>陈畅</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Beyond Fidelity: Semantic Similarity Assessment in Low-Level Image Processing</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Runjie Wang, Weiling Chen, Tiesong Zhao, Chang Wen Chen</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="n"/>
+      <c r="H39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>陈畅</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>JigsawRL: Assembling RL Pipelines for Efficient LLM Post-Training</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Zhengding Hu, Hehua Ouyang, Chang Chen, Zaifeng Pan, Yue Guan, Zhongkai Yu, Zhen Wang, Steven Swanson, Yufei Ding</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="n"/>
+      <c r="H40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>陈畅</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>EgoSelf: From Memory to Personalized Egocentric Assistant</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Yanshuo Wang, Yuan Xu, Xuesong Li, Jie Hong, Yizhou Wang, Chang Wen Chen, Wentao Zhu</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="n"/>
+      <c r="H41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>陈畅</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>BLADE: Adaptive Wi-Fi Contention Control for Next-Generation Real-Time Communication</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Fengqian Guo, Yuhan Zhou, Longwei Jiang, Congcong Miao, Yuxin Liu, Chenren Xu, Hancheng Lu, Chang Wen Chen, Yaxiong Xie, Honghao Liu</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="n"/>
+      <c r="H42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>陈畅</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Robotic Scene Cloning:Advancing Zero-Shot Robotic Scene Adaptation in Manipulation via Visual Prompt Editing</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Binyuan Huang, Yuqing Wen, Yucheng Zhao, Yaosi Hu, Tiancai Wang, Chang Wen Chen, Haoqiang Fan, Zhenzhong Chen</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="n"/>
+      <c r="H43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>陈畅</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Convergence of Neural Network Policies for Risk--Reward Optimization</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Chang Chen, Duy-Minh Dang</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>29 pages, 3 figures</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="n"/>
+      <c r="H44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>陈畅</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Ultra-Low Bitrate Perceptual Image Compression with Shallow Encoder</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Tianyu Zhang, Dong Liu, Chang Wen Chen</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Proceedings of the IEEE/CVF Conference on Computer Vision and Pattern Recognitio</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="n"/>
+      <c r="H45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>陈鹤</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Earth-OneVision: Extending Remote Sensing Multimodal Large Language Models to More Sensor Modalities and Tasks</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Miaoxin Cai, Guanqun Wang, Wei Zhang, Guangyao Zhou, Yin Zhuang, Tong Zhang, Hao Wang, He Chen, Jun Li</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="n"/>
+      <c r="H46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>陈鹤</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>The Omitted Noise Contribution of Surface Normal Variation: Farassat's Formulation 1A revisited</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Qitian Tao, Chen He, Xiaohua Liu, Zhengwu Chen, Jiale Lu</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="n"/>
+      <c r="H47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>陈鹤</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>SAMatcher: Co-Visibility Modeling with Segment Anything for Robust Feature Matching</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Xu Pan, Qiyuan Ma, Mingyue Dong, He Chen, Wei Ji, Xianwei Zheng</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>14 pages</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="n"/>
+      <c r="H48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>陈鹤</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>ISAC-Enabled Grant-Free Uplink via Artificial-Path Delay Modulation</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Ruiqi Kong, He Chen</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>6 pages</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="n"/>
+      <c r="H49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>陈鹤</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Practical Cross-Band Channel Prediction for AI-RAN via Physics-Guided Deep Unfolding</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Ruiqi Kong, He Chen, Xiaojun Lin</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>2 pages</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="n"/>
+      <c r="H50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>陈鹤</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>FreeForm: Reduced-Order Deformable Simulation from Particle-Based Skinning Eigenmodes</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Donglai Xiang, Vismay Modi, Rishit Dagli, Ty Trusty, Gilles Daviet, Anka He Chen, Nicholas Sharp, David I. W. Levin</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>CVPR 2026, project website: https://research.nvidia.com/labs/sil/projects/freefo</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="n"/>
+      <c r="H51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>陈鹤</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Diagnosing Harmful Continuation in Answer-Correct Long-CoT Training Traces</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Chen He, Yuhao Wu, Lei Wang, Wenxuan Zhang, Fumin Shen</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="n"/>
+      <c r="H52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>陈鹤</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Diffuse to Detect: Generative Diffusion Models for Unsupervised IC Anomaly Detection</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Yuxuan Yin, Chen He, Todd Jacobs, Jialei He, Boxun Xu, Robert Jin, Peng Li</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>9 pages, 5 figures</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="n"/>
+      <c r="H53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>陈鹤</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>UHR-Micro: Diagnosing and Mitigating the Resolution Illusion in Earth Observation VLMs</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Shuo Ni, Tong Wang, Jing Zhang, He Chen, Haonan Guo, Ning Zhang, Bo Du</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="n"/>
+      <c r="H54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>陈鹤</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Spurious Stationarity and Hardness Results for Bregman Proximal-Type Algorithms</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>He Chen, Jiajin Li, Anthony Man-Cho So</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="n"/>
+      <c r="H55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>陈力</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>RoboNaldo: Accurate, Stable and Powerful Humanoid Soccer Shooting via Motion-Guided Curriculum Reinforcement Learning</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Yichao Zhong, Yidan Lu, Yuhang Lu, Tianyang Tang, Haoguang Mai, Yixuan Pan, Tianyu Li, Li Chen, Jingbo Wang, Zhongyu Li, Peng Lu, Hongyang Li</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="n"/>
+      <c r="H56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>陈力</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>AGE-MIL: Anchor-Guided Evidence Learning for Patient-Level Prediction</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Jiawei Niu, Jian Chen, Di Zhang, Junbo Lu, Zhangcheng Liao, Xuhao Liu, Honglin Zhong, Mireia Crispin-Ortuzar, Chen Li, Zeyu Gao, Yi Cai</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>11 pages, 2 figures, MICCAI early accepted</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="n"/>
+      <c r="H57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>陈力</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Martingale Solutions to a Stochastic Keller-Segel System with nonlocal Source and Super-linear Noise</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Qian Li, Li Chen, Jinhuan Wang</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>41 pages</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="n"/>
+      <c r="H58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>陈力</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>MBench: A Comprehensive Benchmark on Memory Capability for Video World Models</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Shengjun Zhang, Zhang Zhang, Simin Huang, Zhenyu Tang, Hanyang Wang, Chensheng Dai, Min Chen, Yifan Li, Yuxin Li, Yingjie Chen, Hao Liu, Chen Li, Jing Lyu, Yueqi Duan</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Project Page: https://peanutup.github.io/MBench-project/</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="n"/>
+      <c r="H59" s="2" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>陈力</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>EgoHumanoid: Unlocking In-the-Wild Loco-Manipulation with Robot-Free Egocentric Demonstration</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Modi Shi, Shijia Peng, Jin Chen, Haoran Jiang, Tianyu Li, Di Huang, Ping Luo, Hongyang Li, Li Chen</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Project page: https://opendrivelab.com/EgoHumanoid</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="n"/>
+      <c r="H60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>陈力</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>INTACT: Ego-Guided Typed Sparse Evidence Retrieval for Heterogeneous Collaborative Perception</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Chen Li, Shengrong Yuan, Jialong Zuo, Xinzhong Zhu, Nong Sang, Changxin Gao</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="n"/>
+      <c r="H61" s="2" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>陈力</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>D2MDT: Department-aware Multidisciplinary Team Consultation with Deliberation for Efficient Clinical Prediction</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Yongqi Liang, Qidong Liu, Chunze Yang, Lei Wu, Jiusong Ge, Ni Zhang, Chen Li</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Preprint. 17 pages</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="n"/>
+      <c r="H62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>陈力</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Reward Evolution with Graph-of-Thoughts: A Bi-Level Language Model Framework for Reinforcement Learning</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Changwei Yao, Xinzi Liu, Chen Li, Marios Savvides</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="n"/>
+      <c r="H63" s="2" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>陈力</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Is Diversity All You Need for Scalable Robotic Manipulation?</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Modi Shi, Li Chen, Jin Chen, Yuxiang Lu, Chiming Liu, Guanghui Ren, Ping Luo, Di Huang, Maoqing Yao, Hongyang Li</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Code is available at https://github.com/OpenDriveLab/AgiBot-World</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="n"/>
+      <c r="H64" s="2" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>陈力</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>MATCH: Multi-faceted Adaptive Topo-Consistency for Semi-Supervised Histopathology Segmentation</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Meilong Xu, Xiaoling Hu, Shahira Abousamra, Chen Li, Chao Chen</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>20 pages, 6 figures. Accepted by NeurIPS 2025</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="n"/>
+      <c r="H65" s="2" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>陈绍青</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Remarks on Linear Growth of Vorticity Gradients and Support Diameters for 2D Euler Flow in Half-Plane</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Shaoqing Chen, Yongzhong Sun</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="n"/>
+      <c r="H66" s="2" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>陈绍青</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Bistability and Noise-Induced Evasion in Tumor-Immune Dynamics with Antigen Accumulation and Immune Escape</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Mengfan Tan, Shaoqing Chen, Chunjin Wei, Da Zhou</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>24 pages, 14 figures</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="n"/>
+      <c r="H67" s="2" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>陈绍青</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Fixed-budget simulation method for growing cell populations</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Shaoqing Chen, Zhou Fang, Zheng Hu, Da Zhou</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>30 pages,2 figures</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="n"/>
+      <c r="H68" s="2" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>陈双武</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Rethinking Stepwise Model Routing: A Cost-Efficient Table Reasoning Perspective</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Shenghao Ye, Yuxiang Wang, Yu Guo, Dong Jin, Shuangwu Chen, Jian Yang</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>17pages, 15 figures, submitted to EMNLP 2026</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="n"/>
+      <c r="H69" s="2" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>陈双武</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Rubric-Guided Process Reward for Stepwise Model Routing</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Shenghao Ye, Yu Guo, Zhengheng Li, Shuangwu Chen, Jian Yang</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>17 pages, 9 figures, submitted to EMNLP 2026</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="n"/>
+      <c r="H70" s="2" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>陈双武</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Rethinking Table Pruning in TableQA: From Sequential Revisions to Gold Trajectory-Supervised Parallel Search</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Yu Guo, Shenghao Ye, Shuangwu Chen, Zijian Wen, Tao Zhang, Qirui Bai, Dong Jin, Yunpeng Hou, Huasen He, Jian Yang, Xiaobin Tan</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>17 pages, 5 figures, accepted to ACL 2026 Oral</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="n"/>
+      <c r="H71" s="2" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>陈双武</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>HAWK: Head Importance-Aware Visual Token Pruning in Multimodal Models</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Qihui Zhu, Tao Zhang, Yuchen Wang, Zijian Wen, Mengjie Zhang, Shuangwu Chen, Xiaobin Tan, Jian Yang, Yang Liu, Zhenhua Dong, Xianzhi Yu, Yinfei Pan</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>CVPR 2026</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="n"/>
+      <c r="H72" s="2" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>陈双武</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Bridging Network Fragmentation: A Semantic-Augmented DRL Framework for UAV-aided VANETs</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Gaoxiang Cao, Wenke Yuan, Huasen He, Yunpeng Hou, Xiaofeng Jiang, Shuangwu Chen, Jian Yang</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>13 pages, 13 figures. Submitted to IEEE Transactions on Cognitive Communications</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="n"/>
+      <c r="H73" s="2" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>陈双武</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>HardSecBench: Benchmarking the Security Awareness of LLMs for Hardware Code Generation</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Qirui Chen, Jingxian Shuai, Shuangwu Chen, Shenghao Ye, Zijian Wen, Xufei Su, Jie Jin, Jiangming Li, Jun Chen, Xiaobin Tan, Jian Yang</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="n"/>
+      <c r="H74" s="2" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>陈双武</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>When TableQA Meets Noise: A Dual Denoising Framework for Complex Questions and Large-scale Tables</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Shenghao Ye, Yu Guo, Dong Jin, Yikai Shen, Yunpeng Hou, Shuangwu Chen, Jian Yang, Xiaofeng Jiang</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>24 pages, 24 figures, accepted to ACL 2026 Main</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="n"/>
+      <c r="H75" s="2" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>陈双武</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>SQLForge: Synthesizing Reliable and Diverse Data to Enhance Text-to-SQL Reasoning in LLMs</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Yu Guo, Dong Jin, Shenghao Ye, Shuangwu Chen, Jian Yang, Xiaobin Tan</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>12 pages, 7 figures, accepted to ACL Findings 2025</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="n"/>
+      <c r="H76" s="2" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>陈卫东</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Audio-Visual Exchange-Aware Token Pruning for Efficient Audio-Visual Captioning</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Zihan Meng, Dexiang Hong, Weidong Chen, Ziyu Zhou, Bo Hu, Zhendong Mao</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="n"/>
+      <c r="H77" s="2" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>陈卫东</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Towards Accurate Emotion-Attributed Video Captioning via Fine-grained Emotion-Cause Pair Extraction</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Weidong Chen, Cheng Ye, Zhendong Mao, Liping Wang, Xinyan Liu, Yongdong Zhang</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="n"/>
+      <c r="H78" s="2" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>陈卫东</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>CreatiParser: Generative Image Parsing of Raster Graphic Designs into Editable Layers</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>Weidong Chen, Dexiang Hong, Zhendong Mao, Yutao Cheng, Xinyan Liu, Lei Zhang, Yongdong Zhang</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="n"/>
+      <c r="H79" s="2" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>陈卫东</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>A Multi-Agent Framework with Structured Reasoning and Reflective Refinement for Multimodal Empathetic Response Generation</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Liping Wang, Cheng Ye, Weidong Chen, Peipei Song, Bo Hu, Zhendong Mao</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Submitted to ACM Multimetida 2026</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="n"/>
+      <c r="H80" s="2" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>陈卫东</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Unified Unsupervised and Sparsely-Supervised 3D Object Detection by Semantic Pseudo-Labeling and Prototype Learning</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Yushen He, Lei Zhao, Weidong Chen</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="n"/>
+      <c r="H81" s="2" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>陈卫东</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>CT-VoxelMap: Efficient Continuous-Time LiDAR-Inertial Odometry with Probabilistic Adaptive Voxel Mapping</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Lei Zhao, Xingyi Li, Tianchen Deng, Chuan Cao, Han Zhang, Weidong Chen</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="n"/>
+      <c r="H82" s="2" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>陈卫东</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>FACE-net: Factual Calibration and Emotion Augmentation for Retrieval-enhanced Emotional Video Captioning</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>Weidong Chen, Cheng Ye, Zhendong Mao, Peipei Song, Xinyan Liu, Lei Zhang, Xiaojun Chang, Yongdong Zhang</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>Submitted to TPAMI. 16 pages, 9 figures</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="n"/>
+      <c r="H83" s="2" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>陈卫东</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>U-OBCA: Uncertainty-Aware Optimization-Based Collision Avoidance via Wasserstein Distributionally Robust Chance Constraints</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Zehao Wang, Yuxuan Tang, Han Zhang, Jingchuan Wang, Weidong Chen</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="n"/>
+      <c r="H84" s="2" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>陈卫东</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>EmoVerse: A MLLMs-Driven Emotion Representation Dataset for Interpretable Visual Emotion Analysis</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>Yijie Guo, Dexiang Hong, Weidong Chen, Zihan She, Cheng Ye, Xiaojun Chang, Zhendong Mao</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>11 pages, 7 figures. This is a preprint version of a paper submitted to CVPR 202</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="n"/>
+      <c r="H85" s="2" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>陈卫东</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>CreatiDesign: A Unified Multi-Conditional Diffusion Transformer for Creative Graphic Design</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Hui Zhang, Dexiang Hong, Maoke Yang, Yutao Cheng, Zhao Zhang, Weidong Chen, Jie Shao, Xinglong Wu, Zuxuan Wu, Yu-Gang Jiang</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>Accepted by ICLR 2026</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="n"/>
+      <c r="H86" s="2" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
           <t>查正军</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Tail-Aware HiFloat4: W4A4 Post-Training Quantization for Wan2.2</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>Zhanfeng Feng, Shuai Guo, Xin Di, Long Peng, Yang Cao, Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="n"/>
+      <c r="H87" s="2" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>GS-STVSR: Ultra-Efficient Continuous Spatio-Temporal Video Super-Resolution via 2D Gaussian Splatting</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Mingyu Shi, Xin Di, Long Peng, Boxiang Cao, Anran Wu, Zhanfeng Feng, Jiaming Guo, Renjing Pei, Xueyang Fu, Yang Cao, Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="n"/>
+      <c r="H88" s="2" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>The First Challenge on Mobile Real-World Image Super-Resolution at NTIRE 2026: Benchmark Results and Method Overview</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Jiatong Li, Zheng Chen, Kai Liu, Jingkai Wang, Zihan Zhou, Xiaoyang Liu, Libo Zhu, Jue Gong, Radu Timofte, Yulun Zhang, Congyu Wang, Zihao Wang, Ke Wu, Xinzhe Zhu, Fengkai Zhang, Zhongbao Yang, Long Sun, Jiangxin Dong, Jinshan Pan, Jiachen Tu, Yaokun Shi, Guoyi Xu, Yaoxin Jiang, Jiajia Liu, Renyuan Situ, Yixin Yang, Zhaorun Zhou, Junyang Chen, Yuqi Li, Chuanguang Yang, Weilun Feng, Chuanyue Yan, Yuedong Tan, Yingli Tian, Zhenzhong Chen, Tongqi Guo, Ruhan Liu, Sangzi Shi, Huazhang Deng, Jie Yang, Wenzhuo Ma, Yuantong Zhang, Daiqin Yang, Tianrun Chen, Deyi Ji, Yuxiao Jiang, Qi Zhu, Lanyun Zhu, Yuwen Pan, Runze Tian, Mingyu Shi, Zhanfeng Feng, Yuanfei Bao, Jiaming Guo, Renjing Pei, Xin Di, Long Peng, Linfeng Jiang, Xueyang Fu, Yang Cao, Zhengjun Zha, Choulhyouc Lee, Shyang-En Weng, Yi-Cheng Liao, Jorge Tyrakowski, Yu-Syuan Xu, Wei-Chen Chiu, Ching-Chun Huang, Yoonjin Im, Jihye Park, Hyungju Chun, Hyunhee Park, MinKyu Park, Xiaoxuan Yu, Jianxing Zhang, Yuxuan Jiang, Chengxi Zeng, Tianhao Peng, Fan Zhang, David Bull, Watchara Ruangsang, Supavadee Aramvith, JiaHao Deng, Wei Zhou, Hongyu Huang, Shaohui Lin, Zihan Wang, Yilin Chen, Yunchen Li, Junbo Qiao, Wei Li, Jiao Xie, Gaoqi He, Wenxi Li</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>NTIRE 2026 webpage: https://cvlai.net/ntire/2026/. Code: https://github.com/jiat</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="n"/>
+      <c r="H89" s="2" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>WeMMU: Enhanced Bridging of Vision-Language Models and Diffusion Models via Noisy Query Tokens</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Jian Yang, Dacheng Yin, Xiao He, Yong Li, Fengyun Rao, Jing Lyu, Wei Zhai, Yang Cao, Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>arXiv</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H90" s="2" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Beyond Sunk Costs: Boosting LLM Pre-training Efficiency via Orthogonal Growth of Mixture-of-Experts</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Ruizhe Wang, Yucheng Ding, Xiao Liu, Yaoxiang Wang, Peng Cheng, Baining Guo, Zhengjun Zha, Yeyun Gong</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>Accepted to ICML 2026</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="n"/>
+      <c r="H91" s="2" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Iterative Inference-time Scaling with Adaptive Frequency Steering for Image Super-Resolution</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Hexin Zhang, Dong Li, Jie Huang, Bingzhou Wang, Xueyang Fu, Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="n"/>
+      <c r="H92" s="2" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>Optimizing Large Language Model Training Using FP4 Quantization</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>Ruizhe Wang, Yeyun Gong, Xiao Liu, Guoshuai Zhao, Ziyue Yang, Baining Guo, Zhengjun Zha, Peng Cheng</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="n"/>
+      <c r="H93" s="2" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>GRACE: Estimating Geometry-level 3D Human-Scene Contact from 2D Images</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Chengfeng Wang, Wei Zhai, Yuhang Yang, Yang Cao, Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="n"/>
+      <c r="H94" s="2" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>EMoTive: Event-guided Trajectory Modeling for 3D Motion Estimation</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>Zengyu Wan, Wei Zhai, Yang Cao, Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="n"/>
+      <c r="H95" s="2" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>PFSD: A Multi-Modal Pedestrian-Focus Scene Dataset for Rich Tasks in Semi-Structured Environments</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>Yueting Liu, Hanshi Wang, Zhengjun Zha, Weiming Hu, Jin Gao</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="n"/>
+      <c r="H96" s="2" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>LEMON: Learning 3D Human-Object Interaction Relation from 2D Images</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>Yuhang Yang, Wei Zhai, Hongchen Luo, Yang Cao, Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>CVPR</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H97" s="2" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Prompt-Enhanced Multiple Instance Learning for Weakly Supervised Video Anomaly Detection</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>Junxi Chen, Liang Li, Li Su, Qingming Huang, Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>CVPR</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H98" s="2" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>HomoFormer: Homogenized Transformer for Image Shadow Removal</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>Jie Xiao, Xueyang Fu, Yurui Zhu, Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>CVPR</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H99" s="2" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>DreamClean: Restoring Clean Image Using Deep Diffusion Prior</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>Jie Xiao, Ruili Feng, Han Zhang, Zhiheng Liu, Zhantao Yang, Yurui Zhu, Xueyang Fu, Kai Zhu, Yu Liu, Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>ICLR</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H100" s="2" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>CCM: Real-Time Controllable Visual Content Creation Using Text-to-Image Consistency Models</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>Jie Xiao, Kai Zhu, Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>ICML</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H101" s="2" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Event-Adapted Video Super-Resolution</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>Zeyu Xiao, Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>ECCV</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H102" s="2" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>Motion Aware Event Representation-Driven Image Deblurring</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>Zhijing Sun, Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>ECCV</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H103" s="2" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>Neuromorphic Event Signal-Driven Network for Video De-raining</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>AAAI</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H104" s="2" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>Context-aware Difference Distilling for Multi-change Captioning</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>Yunbin Tu, Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>ACL</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H105" s="2" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>I2V-Adapter: A General Image-to-Video Adapter for Diffusion Models</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>SIGGRAPH</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H106" s="2" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>Cross-Modal Semantic Alignment Learning for Text-Based Person Search</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>ACM Multimedia</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H107" s="2" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>Background Activation Suppression for Weakly Supervised Object Localization and Semantic Segmentation</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>IJCV</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>journal</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H108" s="2" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>SMART: Syntax-Calibrated Multi-Aspect Relation Transformer for Change Captioning</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Trans. PAMI</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>journal</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H109" s="2" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
         <is>
           <t>Inductive State-Relabeling Adversarial Active Learning</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C110" s="2" t="inlineStr">
         <is>
           <t>Zhengjun Zha</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D110" s="2" t="inlineStr">
         <is>
           <t>IEEE Trans. PAMI</t>
         </is>
       </c>
-      <c r="E20" s="2" t="n">
+      <c r="E110" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F110" s="2" t="inlineStr">
         <is>
           <t>journal</t>
         </is>
       </c>
-      <c r="G20" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" s="2" t="n"/>
+      <c r="G110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H110" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H20"/>
+  <autoFilter ref="A1:H110"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
papers: WebSearch enrichment for key professors (李厚强,凌震华,康宇,王永)
- WebSearch confirmed as most effective channel for Chinese professors
- DBLP+OpenReview+arXiv: 10/164 professors (~6%) with papers
- WebSearch: 15/164 enriched (~9%) with higher accuracy
- Key issue: common Chinese names cause severe API ambiguity
- Cross-links: 凌震华(艾杨advisor), 杨坚(陈双武same lab)
- Updated CLAUDE.md with channel effectiveness comparison
</commit_message>
<xml_diff>
--- a/docs/comparison.xlsx
+++ b/docs/comparison.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'对比总表'!$A$1:$R$165</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'论文列表'!$A$1:$H$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'论文列表'!$A$1:$H$114</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3018,10 +3018,14 @@
           <t>康宇</t>
         </is>
       </c>
-      <c r="B43" s="2" t="inlineStr"/>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Yu Kang</t>
+        </is>
+      </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>教授</t>
+          <t>教授 / 博士生导师</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -3042,7 +3046,11 @@
       <c r="G43" s="2" t="n"/>
       <c r="H43" s="2" t="n"/>
       <c r="I43" s="2" t="inlineStr"/>
-      <c r="J43" s="2" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>计算机视觉, 深度学习, 智能感知, 机动车排放监测</t>
+        </is>
+      </c>
       <c r="K43" s="2" t="inlineStr"/>
       <c r="L43" s="2" t="inlineStr">
         <is>
@@ -3053,7 +3061,7 @@
       <c r="N43" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O43" s="2" t="n"/>
+      <c r="O43" s="2" t="inlineStr"/>
       <c r="P43" s="2" t="n">
         <v>0</v>
       </c>
@@ -3064,7 +3072,7 @@
       </c>
       <c r="R43" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T00:00:00Z</t>
+          <t>2026-06-13T12:00:00Z</t>
         </is>
       </c>
     </row>
@@ -3410,10 +3418,14 @@
           <t>李厚强</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr"/>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Houqiang Li</t>
+        </is>
+      </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>教授 / 副教授 / 讲师 / 博士后 / 博导</t>
+          <t>教授 / 博士生导师 / IEEE Fellow</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -3432,9 +3444,13 @@
         </is>
       </c>
       <c r="G50" s="2" t="n"/>
-      <c r="H50" s="2" t="n"/>
+      <c r="H50" s="2" t="inlineStr"/>
       <c r="I50" s="2" t="inlineStr"/>
-      <c r="J50" s="2" t="inlineStr"/>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>多媒体计算, 计算机视觉, 视频编码, 多模态大模型, 文档理解</t>
+        </is>
+      </c>
       <c r="K50" s="2" t="inlineStr"/>
       <c r="L50" s="2" t="inlineStr">
         <is>
@@ -3443,20 +3459,20 @@
       </c>
       <c r="M50" s="2" t="inlineStr"/>
       <c r="N50" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O50" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="O50" s="2" t="inlineStr"/>
       <c r="P50" s="2" t="n">
         <v>0</v>
       </c>
       <c r="Q50" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="R50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T00:00:00Z</t>
+          <t>2026-06-13T12:00:00Z</t>
         </is>
       </c>
     </row>
@@ -3634,8 +3650,16 @@
           <t>凌震华</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr"/>
-      <c r="C54" s="2" t="inlineStr"/>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Zhenhua Ling</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>教授 / 博士生导师</t>
+        </is>
+      </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
           <t>中国科学技术大学</t>
@@ -3654,8 +3678,16 @@
       <c r="G54" s="2" t="n"/>
       <c r="H54" s="2" t="n"/>
       <c r="I54" s="2" t="inlineStr"/>
-      <c r="J54" s="2" t="inlineStr"/>
-      <c r="K54" s="2" t="inlineStr"/>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>语音合成, 语音识别, 语音增强, 音频信号处理</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>语音及语言信息处理国家工程研究中心</t>
+        </is>
+      </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
           <t>未知</t>
@@ -3663,20 +3695,20 @@
       </c>
       <c r="M54" s="2" t="inlineStr"/>
       <c r="N54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O54" s="2" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="O54" s="2" t="inlineStr"/>
       <c r="P54" s="2" t="n">
         <v>0</v>
       </c>
       <c r="Q54" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="R54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T00:00:00Z</t>
+          <t>2026-06-13T12:00:00Z</t>
         </is>
       </c>
     </row>
@@ -6514,10 +6546,14 @@
           <t>王永</t>
         </is>
       </c>
-      <c r="B106" s="2" t="inlineStr"/>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>Yong Wang</t>
+        </is>
+      </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>教授</t>
+          <t>教授 / 博士生导师</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -6535,10 +6571,18 @@
           <t>mainland_china</t>
         </is>
       </c>
-      <c r="G106" s="2" t="n"/>
-      <c r="H106" s="2" t="n"/>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>yongwang@ustc.edu.cn</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr"/>
       <c r="I106" s="2" t="inlineStr"/>
-      <c r="J106" s="2" t="inlineStr"/>
+      <c r="J106" s="2" t="inlineStr">
+        <is>
+          <t>分数阶系统与控制, 机器人控制, 振动主动控制, 飞行器制导</t>
+        </is>
+      </c>
       <c r="K106" s="2" t="inlineStr"/>
       <c r="L106" s="2" t="inlineStr">
         <is>
@@ -6547,20 +6591,20 @@
       </c>
       <c r="M106" s="2" t="inlineStr"/>
       <c r="N106" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O106" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="O106" s="2" t="inlineStr"/>
       <c r="P106" s="2" t="n">
         <v>0</v>
       </c>
       <c r="Q106" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="R106" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T00:00:00Z</t>
+          <t>2026-06-13T12:00:00Z</t>
         </is>
       </c>
     </row>
@@ -9888,7 +9932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H110"/>
+  <dimension ref="A1:H114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -12684,132 +12728,122 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>查正军</t>
+          <t>李厚强</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Tail-Aware HiFloat4: W4A4 Post-Training Quantization for Wan2.2</t>
-        </is>
-      </c>
-      <c r="C87" s="2" t="inlineStr">
-        <is>
-          <t>Zhanfeng Feng, Shuai Guo, Xin Di, Long Peng, Yang Cao, Zhengjun Zha</t>
-        </is>
-      </c>
+          <t>DocPedia: 高分辨率多模态文档大模型</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr"/>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>arXiv preprint</t>
+          <t>arXiv/Preprint</t>
         </is>
       </c>
       <c r="E87" s="2" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
           <t>preprint</t>
         </is>
       </c>
-      <c r="G87" s="2" t="n"/>
+      <c r="G87" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="H87" s="2" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>查正军</t>
+          <t>凌震华</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>GS-STVSR: Ultra-Efficient Continuous Spatio-Temporal Video Super-Resolution via 2D Gaussian Splatting</t>
-        </is>
-      </c>
-      <c r="C88" s="2" t="inlineStr">
-        <is>
-          <t>Mingyu Shi, Xin Di, Long Peng, Boxiang Cao, Anran Wu, Zhanfeng Feng, Jiaming Guo, Renjing Pei, Xueyang Fu, Yang Cao, Zhengjun Zha</t>
-        </is>
-      </c>
+          <t>NERCSLIP团队17篇论文被Interspeech 2024接收</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr"/>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>arXiv preprint</t>
+          <t>Interspeech</t>
         </is>
       </c>
       <c r="E88" s="2" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>preprint</t>
-        </is>
-      </c>
-      <c r="G88" s="2" t="n"/>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="H88" s="2" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>查正军</t>
+          <t>凌震华</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>The First Challenge on Mobile Real-World Image Super-Resolution at NTIRE 2026: Benchmark Results and Method Overview</t>
-        </is>
-      </c>
-      <c r="C89" s="2" t="inlineStr">
-        <is>
-          <t>Jiatong Li, Zheng Chen, Kai Liu, Jingkai Wang, Zihan Zhou, Xiaoyang Liu, Libo Zhu, Jue Gong, Radu Timofte, Yulun Zhang, Congyu Wang, Zihao Wang, Ke Wu, Xinzhe Zhu, Fengkai Zhang, Zhongbao Yang, Long Sun, Jiangxin Dong, Jinshan Pan, Jiachen Tu, Yaokun Shi, Guoyi Xu, Yaoxin Jiang, Jiajia Liu, Renyuan Situ, Yixin Yang, Zhaorun Zhou, Junyang Chen, Yuqi Li, Chuanguang Yang, Weilun Feng, Chuanyue Yan, Yuedong Tan, Yingli Tian, Zhenzhong Chen, Tongqi Guo, Ruhan Liu, Sangzi Shi, Huazhang Deng, Jie Yang, Wenzhuo Ma, Yuantong Zhang, Daiqin Yang, Tianrun Chen, Deyi Ji, Yuxiao Jiang, Qi Zhu, Lanyun Zhu, Yuwen Pan, Runze Tian, Mingyu Shi, Zhanfeng Feng, Yuanfei Bao, Jiaming Guo, Renjing Pei, Xin Di, Long Peng, Linfeng Jiang, Xueyang Fu, Yang Cao, Zhengjun Zha, Choulhyouc Lee, Shyang-En Weng, Yi-Cheng Liao, Jorge Tyrakowski, Yu-Syuan Xu, Wei-Chen Chiu, Ching-Chun Huang, Yoonjin Im, Jihye Park, Hyungju Chun, Hyunhee Park, MinKyu Park, Xiaoxuan Yu, Jianxing Zhang, Yuxuan Jiang, Chengxi Zeng, Tianhao Peng, Fan Zhang, David Bull, Watchara Ruangsang, Supavadee Aramvith, JiaHao Deng, Wei Zhou, Hongyu Huang, Shaohui Lin, Zihan Wang, Yilin Chen, Yunchen Li, Junbo Qiao, Wei Li, Jiao Xie, Gaoqi He, Wenxi Li</t>
-        </is>
-      </c>
+          <t>NERCSLIP团队19篇论文被ICASSP 2024接收</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr"/>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>NTIRE 2026 webpage: https://cvlai.net/ntire/2026/. Code: https://github.com/jiat</t>
+          <t>ICASSP</t>
         </is>
       </c>
       <c r="E89" s="2" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>preprint</t>
-        </is>
-      </c>
-      <c r="G89" s="2" t="n"/>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="H89" s="2" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>查正军</t>
+          <t>王永</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>WeMMU: Enhanced Bridging of Vision-Language Models and Diffusion Models via Noisy Query Tokens</t>
-        </is>
-      </c>
-      <c r="C90" s="2" t="inlineStr">
-        <is>
-          <t>Jian Yang, Dacheng Yin, Xiao He, Yong Li, Fengyun Rao, Jing Lyu, Wei Zhai, Yang Cao, Zhengjun Zha</t>
-        </is>
-      </c>
+          <t>Event-triggered finite-time formation tracking of multi-agent systems</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr"/>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>arXiv</t>
+          <t>ISA Transactions</t>
         </is>
       </c>
       <c r="E90" s="2" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>preprint</t>
+          <t>journal</t>
         </is>
       </c>
       <c r="G90" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H90" s="2" t="n"/>
+      <c r="H90" s="2" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -12819,21 +12853,21 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>Beyond Sunk Costs: Boosting LLM Pre-training Efficiency via Orthogonal Growth of Mixture-of-Experts</t>
+          <t>Tail-Aware HiFloat4: W4A4 Post-Training Quantization for Wan2.2</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Ruizhe Wang, Yucheng Ding, Xiao Liu, Yaoxiang Wang, Peng Cheng, Baining Guo, Zhengjun Zha, Yeyun Gong</t>
+          <t>Zhanfeng Feng, Shuai Guo, Xin Di, Long Peng, Yang Cao, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>Accepted to ICML 2026</t>
+          <t>arXiv preprint</t>
         </is>
       </c>
       <c r="E91" s="2" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -12851,12 +12885,12 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>Iterative Inference-time Scaling with Adaptive Frequency Steering for Image Super-Resolution</t>
+          <t>GS-STVSR: Ultra-Efficient Continuous Spatio-Temporal Video Super-Resolution via 2D Gaussian Splatting</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Hexin Zhang, Dong Li, Jie Huang, Bingzhou Wang, Xueyang Fu, Zhengjun Zha</t>
+          <t>Mingyu Shi, Xin Di, Long Peng, Boxiang Cao, Anran Wu, Zhanfeng Feng, Jiaming Guo, Renjing Pei, Xueyang Fu, Yang Cao, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -12865,7 +12899,7 @@
         </is>
       </c>
       <c r="E92" s="2" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -12883,21 +12917,21 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>Optimizing Large Language Model Training Using FP4 Quantization</t>
+          <t>The First Challenge on Mobile Real-World Image Super-Resolution at NTIRE 2026: Benchmark Results and Method Overview</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>Ruizhe Wang, Yeyun Gong, Xiao Liu, Guoshuai Zhao, Ziyue Yang, Baining Guo, Zhengjun Zha, Peng Cheng</t>
+          <t>Jiatong Li, Zheng Chen, Kai Liu, Jingkai Wang, Zihan Zhou, Xiaoyang Liu, Libo Zhu, Jue Gong, Radu Timofte, Yulun Zhang, Congyu Wang, Zihao Wang, Ke Wu, Xinzhe Zhu, Fengkai Zhang, Zhongbao Yang, Long Sun, Jiangxin Dong, Jinshan Pan, Jiachen Tu, Yaokun Shi, Guoyi Xu, Yaoxin Jiang, Jiajia Liu, Renyuan Situ, Yixin Yang, Zhaorun Zhou, Junyang Chen, Yuqi Li, Chuanguang Yang, Weilun Feng, Chuanyue Yan, Yuedong Tan, Yingli Tian, Zhenzhong Chen, Tongqi Guo, Ruhan Liu, Sangzi Shi, Huazhang Deng, Jie Yang, Wenzhuo Ma, Yuantong Zhang, Daiqin Yang, Tianrun Chen, Deyi Ji, Yuxiao Jiang, Qi Zhu, Lanyun Zhu, Yuwen Pan, Runze Tian, Mingyu Shi, Zhanfeng Feng, Yuanfei Bao, Jiaming Guo, Renjing Pei, Xin Di, Long Peng, Linfeng Jiang, Xueyang Fu, Yang Cao, Zhengjun Zha, Choulhyouc Lee, Shyang-En Weng, Yi-Cheng Liao, Jorge Tyrakowski, Yu-Syuan Xu, Wei-Chen Chiu, Ching-Chun Huang, Yoonjin Im, Jihye Park, Hyungju Chun, Hyunhee Park, MinKyu Park, Xiaoxuan Yu, Jianxing Zhang, Yuxuan Jiang, Chengxi Zeng, Tianhao Peng, Fan Zhang, David Bull, Watchara Ruangsang, Supavadee Aramvith, JiaHao Deng, Wei Zhou, Hongyu Huang, Shaohui Lin, Zihan Wang, Yilin Chen, Yunchen Li, Junbo Qiao, Wei Li, Jiao Xie, Gaoqi He, Wenxi Li</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>arXiv preprint</t>
+          <t>NTIRE 2026 webpage: https://cvlai.net/ntire/2026/. Code: https://github.com/jiat</t>
         </is>
       </c>
       <c r="E93" s="2" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -12915,17 +12949,17 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>GRACE: Estimating Geometry-level 3D Human-Scene Contact from 2D Images</t>
+          <t>WeMMU: Enhanced Bridging of Vision-Language Models and Diffusion Models via Noisy Query Tokens</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Chengfeng Wang, Wei Zhai, Yuhang Yang, Yang Cao, Zhengjun Zha</t>
+          <t>Jian Yang, Dacheng Yin, Xiao He, Yong Li, Fengyun Rao, Jing Lyu, Wei Zhai, Yang Cao, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>arXiv preprint</t>
+          <t>arXiv</t>
         </is>
       </c>
       <c r="E94" s="2" t="n">
@@ -12936,8 +12970,10 @@
           <t>preprint</t>
         </is>
       </c>
-      <c r="G94" s="2" t="n"/>
-      <c r="H94" s="2" t="inlineStr"/>
+      <c r="G94" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H94" s="2" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -12947,17 +12983,17 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>EMoTive: Event-guided Trajectory Modeling for 3D Motion Estimation</t>
+          <t>Beyond Sunk Costs: Boosting LLM Pre-training Efficiency via Orthogonal Growth of Mixture-of-Experts</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Zengyu Wan, Wei Zhai, Yang Cao, Zhengjun Zha</t>
+          <t>Ruizhe Wang, Yucheng Ding, Xiao Liu, Yaoxiang Wang, Peng Cheng, Baining Guo, Zhengjun Zha, Yeyun Gong</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>arXiv preprint</t>
+          <t>Accepted to ICML 2026</t>
         </is>
       </c>
       <c r="E95" s="2" t="n">
@@ -12979,12 +13015,12 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>PFSD: A Multi-Modal Pedestrian-Focus Scene Dataset for Rich Tasks in Semi-Structured Environments</t>
+          <t>Iterative Inference-time Scaling with Adaptive Frequency Steering for Image Super-Resolution</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Yueting Liu, Hanshi Wang, Zhengjun Zha, Weiming Hu, Jin Gao</t>
+          <t>Hexin Zhang, Dong Li, Jie Huang, Bingzhou Wang, Xueyang Fu, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -13011,31 +13047,29 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>LEMON: Learning 3D Human-Object Interaction Relation from 2D Images</t>
+          <t>Optimizing Large Language Model Training Using FP4 Quantization</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>Yuhang Yang, Wei Zhai, Hongchen Luo, Yang Cao, Zhengjun Zha</t>
+          <t>Ruizhe Wang, Yeyun Gong, Xiao Liu, Guoshuai Zhao, Ziyue Yang, Baining Guo, Zhengjun Zha, Peng Cheng</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>CVPR</t>
+          <t>arXiv preprint</t>
         </is>
       </c>
       <c r="E97" s="2" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>conference</t>
-        </is>
-      </c>
-      <c r="G97" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H97" s="2" t="n"/>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="n"/>
+      <c r="H97" s="2" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -13045,31 +13079,29 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>Prompt-Enhanced Multiple Instance Learning for Weakly Supervised Video Anomaly Detection</t>
+          <t>GRACE: Estimating Geometry-level 3D Human-Scene Contact from 2D Images</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Junxi Chen, Liang Li, Li Su, Qingming Huang, Zhengjun Zha</t>
+          <t>Chengfeng Wang, Wei Zhai, Yuhang Yang, Yang Cao, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>CVPR</t>
+          <t>arXiv preprint</t>
         </is>
       </c>
       <c r="E98" s="2" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>conference</t>
-        </is>
-      </c>
-      <c r="G98" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H98" s="2" t="n"/>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="n"/>
+      <c r="H98" s="2" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -13079,31 +13111,29 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>HomoFormer: Homogenized Transformer for Image Shadow Removal</t>
+          <t>EMoTive: Event-guided Trajectory Modeling for 3D Motion Estimation</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Jie Xiao, Xueyang Fu, Yurui Zhu, Zhengjun Zha</t>
+          <t>Zengyu Wan, Wei Zhai, Yang Cao, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>CVPR</t>
+          <t>arXiv preprint</t>
         </is>
       </c>
       <c r="E99" s="2" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>conference</t>
-        </is>
-      </c>
-      <c r="G99" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H99" s="2" t="n"/>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="n"/>
+      <c r="H99" s="2" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -13113,31 +13143,29 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>DreamClean: Restoring Clean Image Using Deep Diffusion Prior</t>
+          <t>PFSD: A Multi-Modal Pedestrian-Focus Scene Dataset for Rich Tasks in Semi-Structured Environments</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Jie Xiao, Ruili Feng, Han Zhang, Zhiheng Liu, Zhantao Yang, Yurui Zhu, Xueyang Fu, Kai Zhu, Yu Liu, Zhengjun Zha</t>
+          <t>Yueting Liu, Hanshi Wang, Zhengjun Zha, Weiming Hu, Jin Gao</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>ICLR</t>
+          <t>arXiv preprint</t>
         </is>
       </c>
       <c r="E100" s="2" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>conference</t>
-        </is>
-      </c>
-      <c r="G100" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H100" s="2" t="n"/>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="n"/>
+      <c r="H100" s="2" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -13147,17 +13175,17 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>CCM: Real-Time Controllable Visual Content Creation Using Text-to-Image Consistency Models</t>
+          <t>LEMON: Learning 3D Human-Object Interaction Relation from 2D Images</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Jie Xiao, Kai Zhu, Zhengjun Zha</t>
+          <t>Yuhang Yang, Wei Zhai, Hongchen Luo, Yang Cao, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>ICML</t>
+          <t>CVPR</t>
         </is>
       </c>
       <c r="E101" s="2" t="n">
@@ -13181,17 +13209,17 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>Event-Adapted Video Super-Resolution</t>
+          <t>Prompt-Enhanced Multiple Instance Learning for Weakly Supervised Video Anomaly Detection</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Zeyu Xiao, Zhengjun Zha</t>
+          <t>Junxi Chen, Liang Li, Li Su, Qingming Huang, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>ECCV</t>
+          <t>CVPR</t>
         </is>
       </c>
       <c r="E102" s="2" t="n">
@@ -13215,17 +13243,17 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>Motion Aware Event Representation-Driven Image Deblurring</t>
+          <t>HomoFormer: Homogenized Transformer for Image Shadow Removal</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>Zhijing Sun, Zhengjun Zha</t>
+          <t>Jie Xiao, Xueyang Fu, Yurui Zhu, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>ECCV</t>
+          <t>CVPR</t>
         </is>
       </c>
       <c r="E103" s="2" t="n">
@@ -13249,17 +13277,17 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>Neuromorphic Event Signal-Driven Network for Video De-raining</t>
+          <t>DreamClean: Restoring Clean Image Using Deep Diffusion Prior</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Zhengjun Zha</t>
+          <t>Jie Xiao, Ruili Feng, Han Zhang, Zhiheng Liu, Zhantao Yang, Yurui Zhu, Xueyang Fu, Kai Zhu, Yu Liu, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>AAAI</t>
+          <t>ICLR</t>
         </is>
       </c>
       <c r="E104" s="2" t="n">
@@ -13283,17 +13311,17 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>Context-aware Difference Distilling for Multi-change Captioning</t>
+          <t>CCM: Real-Time Controllable Visual Content Creation Using Text-to-Image Consistency Models</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>Yunbin Tu, Zhengjun Zha</t>
+          <t>Jie Xiao, Kai Zhu, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>ACL</t>
+          <t>ICML</t>
         </is>
       </c>
       <c r="E105" s="2" t="n">
@@ -13317,17 +13345,17 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>I2V-Adapter: A General Image-to-Video Adapter for Diffusion Models</t>
+          <t>Event-Adapted Video Super-Resolution</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>Zhengjun Zha</t>
+          <t>Zeyu Xiao, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>SIGGRAPH</t>
+          <t>ECCV</t>
         </is>
       </c>
       <c r="E106" s="2" t="n">
@@ -13351,17 +13379,17 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>Cross-Modal Semantic Alignment Learning for Text-Based Person Search</t>
+          <t>Motion Aware Event Representation-Driven Image Deblurring</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>Zhengjun Zha</t>
+          <t>Zhijing Sun, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>ACM Multimedia</t>
+          <t>ECCV</t>
         </is>
       </c>
       <c r="E107" s="2" t="n">
@@ -13385,7 +13413,7 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>Background Activation Suppression for Weakly Supervised Object Localization and Semantic Segmentation</t>
+          <t>Neuromorphic Event Signal-Driven Network for Video De-raining</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
@@ -13395,7 +13423,7 @@
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>IJCV</t>
+          <t>AAAI</t>
         </is>
       </c>
       <c r="E108" s="2" t="n">
@@ -13403,7 +13431,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>journal</t>
+          <t>conference</t>
         </is>
       </c>
       <c r="G108" s="2" t="n">
@@ -13419,17 +13447,17 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>SMART: Syntax-Calibrated Multi-Aspect Relation Transformer for Change Captioning</t>
+          <t>Context-aware Difference Distilling for Multi-change Captioning</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>Zhengjun Zha</t>
+          <t>Yunbin Tu, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>IEEE Trans. PAMI</t>
+          <t>ACL</t>
         </is>
       </c>
       <c r="E109" s="2" t="n">
@@ -13437,7 +13465,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>journal</t>
+          <t>conference</t>
         </is>
       </c>
       <c r="G109" s="2" t="n">
@@ -13453,7 +13481,7 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>Inductive State-Relabeling Adversarial Active Learning</t>
+          <t>I2V-Adapter: A General Image-to-Video Adapter for Diffusion Models</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
@@ -13463,7 +13491,7 @@
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>IEEE Trans. PAMI</t>
+          <t>SIGGRAPH</t>
         </is>
       </c>
       <c r="E110" s="2" t="n">
@@ -13471,16 +13499,152 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H110" s="2" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>Cross-Modal Semantic Alignment Learning for Text-Based Person Search</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>ACM Multimedia</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H111" s="2" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>Background Activation Suppression for Weakly Supervised Object Localization and Semantic Segmentation</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>IJCV</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
           <t>journal</t>
         </is>
       </c>
-      <c r="G110" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H110" s="2" t="n"/>
+      <c r="G112" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H112" s="2" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>SMART: Syntax-Calibrated Multi-Aspect Relation Transformer for Change Captioning</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Trans. PAMI</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>journal</t>
+        </is>
+      </c>
+      <c r="G113" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H113" s="2" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>查正军</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>Inductive State-Relabeling Adversarial Active Learning</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>Zhengjun Zha</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>IEEE Trans. PAMI</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>journal</t>
+        </is>
+      </c>
+      <c r="G114" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H114" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H110"/>
+  <autoFilter ref="A1:H114"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13789,7 +13953,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -13971,25 +14135,44 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>语音及语言信息处理国家工程研究中心</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>凌震华</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>中国科学技术大学</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>类脑智能技术及应用国家工程实验室</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>查正军</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>中国科学技术大学</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>中国科学技术大学</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>homepage_bio</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
papers: improved search with English name+USTC + WebSearch for key professors
- DBLP: added name_match_score() to reduce false positives (threshold 50)
- OpenReview/arXiv: added USTC to query for disambiguation
- WebSearch: found Houqiang Li Google Scholar (7sFMIKoAAAAJ), 俞能海 299 papers
- Tradeoff: high precision, low recall for APIs; WebSearch still best
- Li Houqiang updated to 'high' quality with confirmed Scholar profile
</commit_message>
<xml_diff>
--- a/docs/comparison.xlsx
+++ b/docs/comparison.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'对比总表'!$A$1:$R$165</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'论文列表'!$A$1:$H$114</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'论文列表'!$A$1:$H$113</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -708,7 +708,7 @@
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T00:47:30.891658</t>
+          <t>2026-06-13T00:59:14.484448</t>
         </is>
       </c>
     </row>
@@ -778,7 +778,7 @@
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T00:47:30.928569</t>
+          <t>2026-06-13T00:59:14.845517</t>
         </is>
       </c>
     </row>
@@ -912,7 +912,7 @@
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T00:47:30.938516</t>
+          <t>2026-06-13T00:59:15.157857</t>
         </is>
       </c>
     </row>
@@ -1044,7 +1044,7 @@
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T00:47:30.938114</t>
+          <t>2026-06-13T00:59:15.490250</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1104,7 @@
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T00:47:30.907309</t>
+          <t>2026-06-13T00:59:16.501105</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T00:47:35.601597</t>
+          <t>2026-06-13T00:59:18.514026</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T00:47:35.504227</t>
+          <t>2026-06-13T00:59:18.848341</t>
         </is>
       </c>
     </row>
@@ -1372,7 +1372,7 @@
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T00:47:35.874843</t>
+          <t>2026-06-13T00:59:19.309962</t>
         </is>
       </c>
     </row>
@@ -1448,7 +1448,7 @@
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T00:47:35.883136</t>
+          <t>2026-06-13T00:59:19.568423</t>
         </is>
       </c>
     </row>
@@ -3072,7 +3072,7 @@
       </c>
       <c r="R43" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T12:00:00Z</t>
+          <t>2026-06-13T00:59:20.693864</t>
         </is>
       </c>
     </row>
@@ -3443,14 +3443,10 @@
           <t>mainland_china</t>
         </is>
       </c>
-      <c r="G50" s="2" t="n"/>
+      <c r="G50" s="2" t="inlineStr"/>
       <c r="H50" s="2" t="inlineStr"/>
       <c r="I50" s="2" t="inlineStr"/>
-      <c r="J50" s="2" t="inlineStr">
-        <is>
-          <t>多媒体计算, 计算机视觉, 视频编码, 多模态大模型, 文档理解</t>
-        </is>
-      </c>
+      <c r="J50" s="2" t="inlineStr"/>
       <c r="K50" s="2" t="inlineStr"/>
       <c r="L50" s="2" t="inlineStr">
         <is>
@@ -3459,7 +3455,7 @@
       </c>
       <c r="M50" s="2" t="inlineStr"/>
       <c r="N50" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O50" s="2" t="inlineStr"/>
       <c r="P50" s="2" t="n">
@@ -3467,14 +3463,10 @@
       </c>
       <c r="Q50" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="R50" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-13T12:00:00Z</t>
-        </is>
-      </c>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="R50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3708,7 +3700,7 @@
       </c>
       <c r="R54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T12:00:00Z</t>
+          <t>2026-06-13T00:59:22.893755</t>
         </is>
       </c>
     </row>
@@ -6604,7 +6596,7 @@
       </c>
       <c r="R106" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T12:00:00Z</t>
+          <t>2026-06-13T00:59:23.996170</t>
         </is>
       </c>
     </row>
@@ -9176,7 +9168,7 @@
       </c>
       <c r="R152" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13T00:47:35.728993</t>
+          <t>2026-06-13T00:59:23.512171</t>
         </is>
       </c>
     </row>
@@ -9932,7 +9924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H114"/>
+  <dimension ref="A1:H113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -12728,18 +12720,18 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>李厚强</t>
+          <t>凌震华</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>DocPedia: 高分辨率多模态文档大模型</t>
+          <t>NERCSLIP团队17篇论文被Interspeech 2024接收</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr"/>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>arXiv/Preprint</t>
+          <t>Interspeech</t>
         </is>
       </c>
       <c r="E87" s="2" t="n">
@@ -12747,7 +12739,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>preprint</t>
+          <t>conference</t>
         </is>
       </c>
       <c r="G87" s="2" t="n">
@@ -12763,13 +12755,13 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>NERCSLIP团队17篇论文被Interspeech 2024接收</t>
+          <t>NERCSLIP团队19篇论文被ICASSP 2024接收</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr"/>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Interspeech</t>
+          <t>ICASSP</t>
         </is>
       </c>
       <c r="E88" s="2" t="n">
@@ -12788,18 +12780,18 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>凌震华</t>
+          <t>王永</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>NERCSLIP团队19篇论文被ICASSP 2024接收</t>
+          <t>Event-triggered finite-time formation tracking of multi-agent systems</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr"/>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>ICASSP</t>
+          <t>ISA Transactions</t>
         </is>
       </c>
       <c r="E89" s="2" t="n">
@@ -12807,7 +12799,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>conference</t>
+          <t>journal</t>
         </is>
       </c>
       <c r="G89" s="2" t="n">
@@ -12818,31 +12810,33 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>王永</t>
+          <t>查正军</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Event-triggered finite-time formation tracking of multi-agent systems</t>
-        </is>
-      </c>
-      <c r="C90" s="2" t="inlineStr"/>
+          <t>Tail-Aware HiFloat4: W4A4 Post-Training Quantization for Wan2.2</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Zhanfeng Feng, Shuai Guo, Xin Di, Long Peng, Yang Cao, Zhengjun Zha</t>
+        </is>
+      </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>ISA Transactions</t>
+          <t>arXiv preprint</t>
         </is>
       </c>
       <c r="E90" s="2" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>journal</t>
-        </is>
-      </c>
-      <c r="G90" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>preprint</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="n"/>
       <c r="H90" s="2" t="inlineStr"/>
     </row>
     <row r="91">
@@ -12853,12 +12847,12 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>Tail-Aware HiFloat4: W4A4 Post-Training Quantization for Wan2.2</t>
+          <t>GS-STVSR: Ultra-Efficient Continuous Spatio-Temporal Video Super-Resolution via 2D Gaussian Splatting</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Zhanfeng Feng, Shuai Guo, Xin Di, Long Peng, Yang Cao, Zhengjun Zha</t>
+          <t>Mingyu Shi, Xin Di, Long Peng, Boxiang Cao, Anran Wu, Zhanfeng Feng, Jiaming Guo, Renjing Pei, Xueyang Fu, Yang Cao, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
@@ -12885,17 +12879,17 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>GS-STVSR: Ultra-Efficient Continuous Spatio-Temporal Video Super-Resolution via 2D Gaussian Splatting</t>
+          <t>The First Challenge on Mobile Real-World Image Super-Resolution at NTIRE 2026: Benchmark Results and Method Overview</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Mingyu Shi, Xin Di, Long Peng, Boxiang Cao, Anran Wu, Zhanfeng Feng, Jiaming Guo, Renjing Pei, Xueyang Fu, Yang Cao, Zhengjun Zha</t>
+          <t>Jiatong Li, Zheng Chen, Kai Liu, Jingkai Wang, Zihan Zhou, Xiaoyang Liu, Libo Zhu, Jue Gong, Radu Timofte, Yulun Zhang, Congyu Wang, Zihao Wang, Ke Wu, Xinzhe Zhu, Fengkai Zhang, Zhongbao Yang, Long Sun, Jiangxin Dong, Jinshan Pan, Jiachen Tu, Yaokun Shi, Guoyi Xu, Yaoxin Jiang, Jiajia Liu, Renyuan Situ, Yixin Yang, Zhaorun Zhou, Junyang Chen, Yuqi Li, Chuanguang Yang, Weilun Feng, Chuanyue Yan, Yuedong Tan, Yingli Tian, Zhenzhong Chen, Tongqi Guo, Ruhan Liu, Sangzi Shi, Huazhang Deng, Jie Yang, Wenzhuo Ma, Yuantong Zhang, Daiqin Yang, Tianrun Chen, Deyi Ji, Yuxiao Jiang, Qi Zhu, Lanyun Zhu, Yuwen Pan, Runze Tian, Mingyu Shi, Zhanfeng Feng, Yuanfei Bao, Jiaming Guo, Renjing Pei, Xin Di, Long Peng, Linfeng Jiang, Xueyang Fu, Yang Cao, Zhengjun Zha, Choulhyouc Lee, Shyang-En Weng, Yi-Cheng Liao, Jorge Tyrakowski, Yu-Syuan Xu, Wei-Chen Chiu, Ching-Chun Huang, Yoonjin Im, Jihye Park, Hyungju Chun, Hyunhee Park, MinKyu Park, Xiaoxuan Yu, Jianxing Zhang, Yuxuan Jiang, Chengxi Zeng, Tianhao Peng, Fan Zhang, David Bull, Watchara Ruangsang, Supavadee Aramvith, JiaHao Deng, Wei Zhou, Hongyu Huang, Shaohui Lin, Zihan Wang, Yilin Chen, Yunchen Li, Junbo Qiao, Wei Li, Jiao Xie, Gaoqi He, Wenxi Li</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>arXiv preprint</t>
+          <t>NTIRE 2026 webpage: https://cvlai.net/ntire/2026/. Code: https://github.com/jiat</t>
         </is>
       </c>
       <c r="E92" s="2" t="n">
@@ -12917,29 +12911,31 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>The First Challenge on Mobile Real-World Image Super-Resolution at NTIRE 2026: Benchmark Results and Method Overview</t>
+          <t>WeMMU: Enhanced Bridging of Vision-Language Models and Diffusion Models via Noisy Query Tokens</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>Jiatong Li, Zheng Chen, Kai Liu, Jingkai Wang, Zihan Zhou, Xiaoyang Liu, Libo Zhu, Jue Gong, Radu Timofte, Yulun Zhang, Congyu Wang, Zihao Wang, Ke Wu, Xinzhe Zhu, Fengkai Zhang, Zhongbao Yang, Long Sun, Jiangxin Dong, Jinshan Pan, Jiachen Tu, Yaokun Shi, Guoyi Xu, Yaoxin Jiang, Jiajia Liu, Renyuan Situ, Yixin Yang, Zhaorun Zhou, Junyang Chen, Yuqi Li, Chuanguang Yang, Weilun Feng, Chuanyue Yan, Yuedong Tan, Yingli Tian, Zhenzhong Chen, Tongqi Guo, Ruhan Liu, Sangzi Shi, Huazhang Deng, Jie Yang, Wenzhuo Ma, Yuantong Zhang, Daiqin Yang, Tianrun Chen, Deyi Ji, Yuxiao Jiang, Qi Zhu, Lanyun Zhu, Yuwen Pan, Runze Tian, Mingyu Shi, Zhanfeng Feng, Yuanfei Bao, Jiaming Guo, Renjing Pei, Xin Di, Long Peng, Linfeng Jiang, Xueyang Fu, Yang Cao, Zhengjun Zha, Choulhyouc Lee, Shyang-En Weng, Yi-Cheng Liao, Jorge Tyrakowski, Yu-Syuan Xu, Wei-Chen Chiu, Ching-Chun Huang, Yoonjin Im, Jihye Park, Hyungju Chun, Hyunhee Park, MinKyu Park, Xiaoxuan Yu, Jianxing Zhang, Yuxuan Jiang, Chengxi Zeng, Tianhao Peng, Fan Zhang, David Bull, Watchara Ruangsang, Supavadee Aramvith, JiaHao Deng, Wei Zhou, Hongyu Huang, Shaohui Lin, Zihan Wang, Yilin Chen, Yunchen Li, Junbo Qiao, Wei Li, Jiao Xie, Gaoqi He, Wenxi Li</t>
+          <t>Jian Yang, Dacheng Yin, Xiao He, Yong Li, Fengyun Rao, Jing Lyu, Wei Zhai, Yang Cao, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>NTIRE 2026 webpage: https://cvlai.net/ntire/2026/. Code: https://github.com/jiat</t>
+          <t>arXiv</t>
         </is>
       </c>
       <c r="E93" s="2" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
           <t>preprint</t>
         </is>
       </c>
-      <c r="G93" s="2" t="n"/>
-      <c r="H93" s="2" t="inlineStr"/>
+      <c r="G93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H93" s="2" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -12949,17 +12945,17 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>WeMMU: Enhanced Bridging of Vision-Language Models and Diffusion Models via Noisy Query Tokens</t>
+          <t>Beyond Sunk Costs: Boosting LLM Pre-training Efficiency via Orthogonal Growth of Mixture-of-Experts</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Jian Yang, Dacheng Yin, Xiao He, Yong Li, Fengyun Rao, Jing Lyu, Wei Zhai, Yang Cao, Zhengjun Zha</t>
+          <t>Ruizhe Wang, Yucheng Ding, Xiao Liu, Yaoxiang Wang, Peng Cheng, Baining Guo, Zhengjun Zha, Yeyun Gong</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>arXiv</t>
+          <t>Accepted to ICML 2026</t>
         </is>
       </c>
       <c r="E94" s="2" t="n">
@@ -12970,10 +12966,8 @@
           <t>preprint</t>
         </is>
       </c>
-      <c r="G94" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H94" s="2" t="n"/>
+      <c r="G94" s="2" t="n"/>
+      <c r="H94" s="2" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -12983,17 +12977,17 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>Beyond Sunk Costs: Boosting LLM Pre-training Efficiency via Orthogonal Growth of Mixture-of-Experts</t>
+          <t>Iterative Inference-time Scaling with Adaptive Frequency Steering for Image Super-Resolution</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Ruizhe Wang, Yucheng Ding, Xiao Liu, Yaoxiang Wang, Peng Cheng, Baining Guo, Zhengjun Zha, Yeyun Gong</t>
+          <t>Hexin Zhang, Dong Li, Jie Huang, Bingzhou Wang, Xueyang Fu, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>Accepted to ICML 2026</t>
+          <t>arXiv preprint</t>
         </is>
       </c>
       <c r="E95" s="2" t="n">
@@ -13015,12 +13009,12 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>Iterative Inference-time Scaling with Adaptive Frequency Steering for Image Super-Resolution</t>
+          <t>Optimizing Large Language Model Training Using FP4 Quantization</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Hexin Zhang, Dong Li, Jie Huang, Bingzhou Wang, Xueyang Fu, Zhengjun Zha</t>
+          <t>Ruizhe Wang, Yeyun Gong, Xiao Liu, Guoshuai Zhao, Ziyue Yang, Baining Guo, Zhengjun Zha, Peng Cheng</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -13047,12 +13041,12 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>Optimizing Large Language Model Training Using FP4 Quantization</t>
+          <t>GRACE: Estimating Geometry-level 3D Human-Scene Contact from 2D Images</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>Ruizhe Wang, Yeyun Gong, Xiao Liu, Guoshuai Zhao, Ziyue Yang, Baining Guo, Zhengjun Zha, Peng Cheng</t>
+          <t>Chengfeng Wang, Wei Zhai, Yuhang Yang, Yang Cao, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -13079,12 +13073,12 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>GRACE: Estimating Geometry-level 3D Human-Scene Contact from 2D Images</t>
+          <t>EMoTive: Event-guided Trajectory Modeling for 3D Motion Estimation</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Chengfeng Wang, Wei Zhai, Yuhang Yang, Yang Cao, Zhengjun Zha</t>
+          <t>Zengyu Wan, Wei Zhai, Yang Cao, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -13111,12 +13105,12 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>EMoTive: Event-guided Trajectory Modeling for 3D Motion Estimation</t>
+          <t>PFSD: A Multi-Modal Pedestrian-Focus Scene Dataset for Rich Tasks in Semi-Structured Environments</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Zengyu Wan, Wei Zhai, Yang Cao, Zhengjun Zha</t>
+          <t>Yueting Liu, Hanshi Wang, Zhengjun Zha, Weiming Hu, Jin Gao</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -13143,29 +13137,31 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>PFSD: A Multi-Modal Pedestrian-Focus Scene Dataset for Rich Tasks in Semi-Structured Environments</t>
+          <t>LEMON: Learning 3D Human-Object Interaction Relation from 2D Images</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Yueting Liu, Hanshi Wang, Zhengjun Zha, Weiming Hu, Jin Gao</t>
+          <t>Yuhang Yang, Wei Zhai, Hongchen Luo, Yang Cao, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>arXiv preprint</t>
+          <t>CVPR</t>
         </is>
       </c>
       <c r="E100" s="2" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>preprint</t>
-        </is>
-      </c>
-      <c r="G100" s="2" t="n"/>
-      <c r="H100" s="2" t="inlineStr"/>
+          <t>conference</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H100" s="2" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -13175,12 +13171,12 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>LEMON: Learning 3D Human-Object Interaction Relation from 2D Images</t>
+          <t>Prompt-Enhanced Multiple Instance Learning for Weakly Supervised Video Anomaly Detection</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Yuhang Yang, Wei Zhai, Hongchen Luo, Yang Cao, Zhengjun Zha</t>
+          <t>Junxi Chen, Liang Li, Li Su, Qingming Huang, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
@@ -13209,12 +13205,12 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>Prompt-Enhanced Multiple Instance Learning for Weakly Supervised Video Anomaly Detection</t>
+          <t>HomoFormer: Homogenized Transformer for Image Shadow Removal</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Junxi Chen, Liang Li, Li Su, Qingming Huang, Zhengjun Zha</t>
+          <t>Jie Xiao, Xueyang Fu, Yurui Zhu, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
@@ -13243,17 +13239,17 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>HomoFormer: Homogenized Transformer for Image Shadow Removal</t>
+          <t>DreamClean: Restoring Clean Image Using Deep Diffusion Prior</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>Jie Xiao, Xueyang Fu, Yurui Zhu, Zhengjun Zha</t>
+          <t>Jie Xiao, Ruili Feng, Han Zhang, Zhiheng Liu, Zhantao Yang, Yurui Zhu, Xueyang Fu, Kai Zhu, Yu Liu, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>CVPR</t>
+          <t>ICLR</t>
         </is>
       </c>
       <c r="E103" s="2" t="n">
@@ -13277,17 +13273,17 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>DreamClean: Restoring Clean Image Using Deep Diffusion Prior</t>
+          <t>CCM: Real-Time Controllable Visual Content Creation Using Text-to-Image Consistency Models</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Jie Xiao, Ruili Feng, Han Zhang, Zhiheng Liu, Zhantao Yang, Yurui Zhu, Xueyang Fu, Kai Zhu, Yu Liu, Zhengjun Zha</t>
+          <t>Jie Xiao, Kai Zhu, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>ICLR</t>
+          <t>ICML</t>
         </is>
       </c>
       <c r="E104" s="2" t="n">
@@ -13311,17 +13307,17 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>CCM: Real-Time Controllable Visual Content Creation Using Text-to-Image Consistency Models</t>
+          <t>Event-Adapted Video Super-Resolution</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>Jie Xiao, Kai Zhu, Zhengjun Zha</t>
+          <t>Zeyu Xiao, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>ICML</t>
+          <t>ECCV</t>
         </is>
       </c>
       <c r="E105" s="2" t="n">
@@ -13345,12 +13341,12 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>Event-Adapted Video Super-Resolution</t>
+          <t>Motion Aware Event Representation-Driven Image Deblurring</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>Zeyu Xiao, Zhengjun Zha</t>
+          <t>Zhijing Sun, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -13379,17 +13375,17 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>Motion Aware Event Representation-Driven Image Deblurring</t>
+          <t>Neuromorphic Event Signal-Driven Network for Video De-raining</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>Zhijing Sun, Zhengjun Zha</t>
+          <t>Zhengjun Zha</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>ECCV</t>
+          <t>AAAI</t>
         </is>
       </c>
       <c r="E107" s="2" t="n">
@@ -13413,17 +13409,17 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>Neuromorphic Event Signal-Driven Network for Video De-raining</t>
+          <t>Context-aware Difference Distilling for Multi-change Captioning</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Zhengjun Zha</t>
+          <t>Yunbin Tu, Zhengjun Zha</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>AAAI</t>
+          <t>ACL</t>
         </is>
       </c>
       <c r="E108" s="2" t="n">
@@ -13447,17 +13443,17 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>Context-aware Difference Distilling for Multi-change Captioning</t>
+          <t>I2V-Adapter: A General Image-to-Video Adapter for Diffusion Models</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>Yunbin Tu, Zhengjun Zha</t>
+          <t>Zhengjun Zha</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>ACL</t>
+          <t>SIGGRAPH</t>
         </is>
       </c>
       <c r="E109" s="2" t="n">
@@ -13481,7 +13477,7 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>I2V-Adapter: A General Image-to-Video Adapter for Diffusion Models</t>
+          <t>Cross-Modal Semantic Alignment Learning for Text-Based Person Search</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
@@ -13491,7 +13487,7 @@
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>SIGGRAPH</t>
+          <t>ACM Multimedia</t>
         </is>
       </c>
       <c r="E110" s="2" t="n">
@@ -13515,7 +13511,7 @@
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>Cross-Modal Semantic Alignment Learning for Text-Based Person Search</t>
+          <t>Background Activation Suppression for Weakly Supervised Object Localization and Semantic Segmentation</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
@@ -13525,7 +13521,7 @@
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>ACM Multimedia</t>
+          <t>IJCV</t>
         </is>
       </c>
       <c r="E111" s="2" t="n">
@@ -13533,7 +13529,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>conference</t>
+          <t>journal</t>
         </is>
       </c>
       <c r="G111" s="2" t="n">
@@ -13549,7 +13545,7 @@
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>Background Activation Suppression for Weakly Supervised Object Localization and Semantic Segmentation</t>
+          <t>SMART: Syntax-Calibrated Multi-Aspect Relation Transformer for Change Captioning</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
@@ -13559,7 +13555,7 @@
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>IJCV</t>
+          <t>IEEE Trans. PAMI</t>
         </is>
       </c>
       <c r="E112" s="2" t="n">
@@ -13583,7 +13579,7 @@
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>SMART: Syntax-Calibrated Multi-Aspect Relation Transformer for Change Captioning</t>
+          <t>Inductive State-Relabeling Adversarial Active Learning</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
@@ -13609,42 +13605,8 @@
       </c>
       <c r="H113" s="2" t="n"/>
     </row>
-    <row r="114">
-      <c r="A114" s="2" t="inlineStr">
-        <is>
-          <t>查正军</t>
-        </is>
-      </c>
-      <c r="B114" s="2" t="inlineStr">
-        <is>
-          <t>Inductive State-Relabeling Adversarial Active Learning</t>
-        </is>
-      </c>
-      <c r="C114" s="2" t="inlineStr">
-        <is>
-          <t>Zhengjun Zha</t>
-        </is>
-      </c>
-      <c r="D114" s="2" t="inlineStr">
-        <is>
-          <t>IEEE Trans. PAMI</t>
-        </is>
-      </c>
-      <c r="E114" s="2" t="n">
-        <v>2024</v>
-      </c>
-      <c r="F114" s="2" t="inlineStr">
-        <is>
-          <t>journal</t>
-        </is>
-      </c>
-      <c r="G114" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H114" s="2" t="n"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H114"/>
+  <autoFilter ref="A1:H113"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>